<commit_message>
vault backup: 2026-10-30 15:48:02
</commit_message>
<xml_diff>
--- a/02云云天平/03业务模块/HSK3.0/新旧大纲对比(含HSK、HSKK).xlsx
+++ b/02云云天平/03业务模块/HSK3.0/新旧大纲对比(含HSK、HSKK).xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView windowWidth="21615" windowHeight="17655" activeTab="3"/>
+    <workbookView windowWidth="21615" windowHeight="17655" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="HSK新旧大纲对比" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="442" uniqueCount="310">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="442" uniqueCount="311">
   <si>
     <t>HSK1</t>
   </si>
@@ -640,6 +640,9 @@
 3.0：改为逐题准备——三级第 14、15 题各 3 分钟；四~六级看图说话 3 分钟、回答问题 3.5 分钟/题；听后重复/听后复述/看图说话（三级）无准备时间。</t>
   </si>
   <si>
+    <t>写作、书写</t>
+  </si>
+  <si>
     <t>翻译</t>
   </si>
   <si>
@@ -980,6 +983,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10.5"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+      </rPr>
       <t>听一句</t>
     </r>
     <r>
@@ -1048,6 +1057,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10.5"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+      </rPr>
       <t>仅</t>
     </r>
     <r>
@@ -1098,6 +1113,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10.5"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI"/>
+        <charset val="134"/>
+      </rPr>
       <t xml:space="preserve">3.0 </t>
     </r>
     <r>
@@ -1139,6 +1160,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10.5"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI"/>
+        <charset val="134"/>
+      </rPr>
       <t xml:space="preserve">2.0 </t>
     </r>
     <r>
@@ -1252,6 +1279,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10.5"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+      </rPr>
       <t>仅</t>
     </r>
     <r>
@@ -1302,6 +1335,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10.5"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+      </rPr>
       <t>两版均有，恒</t>
     </r>
     <r>
@@ -3677,206 +3716,206 @@
       <c r="E1" s="2"/>
       <c r="F1" s="3"/>
       <c r="G1" s="7" t="s">
-        <v>26</v>
+        <v>176</v>
       </c>
       <c r="H1" s="2"/>
       <c r="I1" s="3"/>
       <c r="J1" s="8" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="K1" s="3"/>
       <c r="L1" s="8" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="M1" s="3"/>
     </row>
     <row r="2" s="6" customFormat="1" ht="28.5" customHeight="1" spans="1:13">
       <c r="A2" s="4" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B2" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="D2" s="4" t="s">
         <v>179</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="E2" s="5" t="s">
         <v>180</v>
       </c>
-      <c r="D2" s="4" t="s">
-        <v>178</v>
-      </c>
-      <c r="E2" s="5" t="s">
+      <c r="F2" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="G2" s="4" t="s">
         <v>179</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="H2" s="5" t="s">
         <v>180</v>
       </c>
-      <c r="G2" s="4" t="s">
-        <v>178</v>
-      </c>
-      <c r="H2" s="5" t="s">
+      <c r="I2" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="J2" s="4" t="s">
         <v>179</v>
       </c>
-      <c r="I2" s="4" t="s">
+      <c r="K2" s="5" t="s">
         <v>180</v>
       </c>
-      <c r="J2" s="4" t="s">
-        <v>178</v>
-      </c>
-      <c r="K2" s="5" t="s">
+      <c r="L2" s="4" t="s">
         <v>179</v>
       </c>
-      <c r="L2" s="4" t="s">
-        <v>178</v>
-      </c>
       <c r="M2" s="9" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
     </row>
     <row r="3" s="6" customFormat="1" ht="15.75" customHeight="1" spans="1:13">
       <c r="A3" s="4" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B3" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="D3" s="4" t="s">
         <v>182</v>
       </c>
-      <c r="C3" s="4" t="s">
-        <v>183</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>181</v>
-      </c>
       <c r="E3" s="4" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="K3" s="4" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="L3" s="5" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="M3" s="10" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
     </row>
     <row r="4" s="6" customFormat="1" ht="47.25" customHeight="1" spans="1:13">
       <c r="A4" s="4" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="J4" s="4" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="K4" s="10" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="L4" s="10" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="M4" s="10" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="5" s="6" customFormat="1" ht="47.25" customHeight="1" spans="1:13">
       <c r="A5" s="4" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="D5" s="4" t="s">
+        <v>209</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>210</v>
+      </c>
+      <c r="F5" s="4" t="s">
         <v>208</v>
       </c>
-      <c r="E5" s="4" t="s">
-        <v>209</v>
-      </c>
-      <c r="F5" s="4" t="s">
-        <v>207</v>
-      </c>
       <c r="G5" s="4" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J5" s="10"/>
       <c r="K5" s="10"/>
       <c r="L5" s="10" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="M5" s="10" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="6" s="6" customFormat="1" ht="47.25" customHeight="1" spans="1:13">
       <c r="A6" s="4" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="J6" s="9"/>
       <c r="K6" s="9"/>
@@ -3885,31 +3924,31 @@
     </row>
     <row r="7" s="6" customFormat="1" ht="31.5" customHeight="1" spans="1:13">
       <c r="A7" s="4" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="I7" s="4" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="J7" s="9"/>
       <c r="K7" s="9"/>
@@ -3918,31 +3957,31 @@
     </row>
     <row r="8" s="6" customFormat="1" ht="47.25" customHeight="1" spans="1:13">
       <c r="A8" s="4" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="I8" s="4" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="J8" s="9"/>
       <c r="K8" s="9"/>
@@ -3951,31 +3990,31 @@
     </row>
     <row r="9" s="6" customFormat="1" ht="15.75" customHeight="1" spans="1:13">
       <c r="A9" s="4" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="I9" s="4" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="J9" s="9"/>
       <c r="K9" s="9"/>
@@ -3984,31 +4023,31 @@
     </row>
     <row r="10" s="6" customFormat="1" ht="31.5" customHeight="1" spans="1:13">
       <c r="A10" s="4" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="I10" s="4" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="J10" s="9"/>
       <c r="K10" s="9"/>
@@ -4017,31 +4056,31 @@
     </row>
     <row r="11" s="6" customFormat="1" ht="31.5" customHeight="1" spans="1:13">
       <c r="A11" s="4" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="I11" s="4" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="J11" s="9"/>
       <c r="K11" s="9"/>
@@ -4050,31 +4089,31 @@
     </row>
     <row r="12" s="6" customFormat="1" ht="47.25" customHeight="1" spans="1:13">
       <c r="A12" s="4" t="s">
+        <v>267</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="C12" s="4" t="s">
         <v>266</v>
       </c>
-      <c r="B12" s="4" t="s">
-        <v>182</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>265</v>
-      </c>
       <c r="D12" s="4" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="G12" s="9" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="H12" s="9" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="I12" s="9" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="J12" s="9"/>
       <c r="K12" s="9"/>
@@ -4083,22 +4122,22 @@
     </row>
     <row r="13" s="6" customFormat="1" ht="31.5" customHeight="1" spans="1:13">
       <c r="A13" s="4" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="G13" s="9"/>
       <c r="H13" s="9"/>
@@ -4113,13 +4152,13 @@
       <c r="B14" s="9"/>
       <c r="C14" s="9"/>
       <c r="D14" s="4" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="G14" s="9"/>
       <c r="H14" s="9"/>
@@ -4134,13 +4173,13 @@
       <c r="B15" s="9"/>
       <c r="C15" s="9"/>
       <c r="D15" s="4" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="G15" s="9"/>
       <c r="H15" s="9"/>
@@ -4155,13 +4194,13 @@
       <c r="B16" s="9"/>
       <c r="C16" s="9"/>
       <c r="D16" s="4" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="G16" s="9"/>
       <c r="H16" s="9"/>
@@ -4198,7 +4237,7 @@
   <sheetData>
     <row r="1" ht="22" customHeight="1" spans="1:4">
       <c r="A1" s="1" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -4206,100 +4245,100 @@
     </row>
     <row r="2" ht="28" customHeight="1" spans="1:4">
       <c r="A2" s="4" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="3" ht="34" customHeight="1" spans="1:4">
       <c r="A3" s="4" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
     </row>
     <row r="4" ht="34" customHeight="1" spans="1:4">
       <c r="A4" s="4" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
     </row>
     <row r="5" ht="34" customHeight="1" spans="1:4">
       <c r="A5" s="4" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
     </row>
     <row r="6" ht="34" customHeight="1" spans="1:4">
       <c r="A6" s="4" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
     </row>
     <row r="7" ht="34" customHeight="1" spans="1:4">
       <c r="A7" s="4" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
     </row>
     <row r="8" ht="34" customHeight="1" spans="1:4">
       <c r="A8" s="4" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
vault backup: 2026-10-30 16:37:54
</commit_message>
<xml_diff>
--- a/02云云天平/03业务模块/HSK3.0/新旧大纲对比(含HSK、HSKK).xlsx
+++ b/02云云天平/03业务模块/HSK3.0/新旧大纲对比(含HSK、HSKK).xlsx
@@ -3173,7 +3173,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G70"/>
+  <dimension ref="A1:G72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3192,7 +3192,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="32" customHeight="1">
+    <row r="2" ht="38" customHeight="1">
       <c r="A2" s="23" t="inlineStr">
         <is>
           <t>模块</t>
@@ -3229,7 +3229,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="21" customHeight="1">
+    <row r="3" ht="23" customHeight="1">
       <c r="A3" s="24" t="inlineStr">
         <is>
           <t>听力</t>
@@ -3266,7 +3266,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="36" customHeight="1">
+    <row r="4" ht="38" customHeight="1">
       <c r="A4" s="24" t="inlineStr">
         <is>
           <t>听力</t>
@@ -3303,7 +3303,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="21" customHeight="1">
+    <row r="5" ht="23" customHeight="1">
       <c r="A5" s="24" t="inlineStr">
         <is>
           <t>听力</t>
@@ -3340,7 +3340,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="36" customHeight="1">
+    <row r="6" ht="38" customHeight="1">
       <c r="A6" s="24" t="inlineStr">
         <is>
           <t>听力</t>
@@ -3377,7 +3377,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="21" customHeight="1">
+    <row r="7" ht="38" customHeight="1">
       <c r="A7" s="24" t="inlineStr">
         <is>
           <t>听力</t>
@@ -3410,7 +3410,7 @@
       </c>
       <c r="G7" s="25" t="inlineStr"/>
     </row>
-    <row r="8" ht="21" customHeight="1">
+    <row r="8" ht="38" customHeight="1">
       <c r="A8" s="24" t="inlineStr">
         <is>
           <t>听力</t>
@@ -3447,7 +3447,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="21" customHeight="1">
+    <row r="9" ht="23" customHeight="1">
       <c r="A9" s="24" t="inlineStr">
         <is>
           <t>听力</t>
@@ -3484,7 +3484,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="21" customHeight="1">
+    <row r="10" ht="23" customHeight="1">
       <c r="A10" s="24" t="inlineStr">
         <is>
           <t>听力</t>
@@ -3517,7 +3517,7 @@
       </c>
       <c r="G10" s="25" t="inlineStr"/>
     </row>
-    <row r="11" ht="21" customHeight="1">
+    <row r="11" ht="23" customHeight="1">
       <c r="A11" s="24" t="inlineStr">
         <is>
           <t>听力</t>
@@ -3554,7 +3554,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="21" customHeight="1">
+    <row r="12" ht="38" customHeight="1">
       <c r="A12" s="24" t="inlineStr">
         <is>
           <t>听力</t>
@@ -3591,7 +3591,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="36" customHeight="1">
+    <row r="13" ht="38" customHeight="1">
       <c r="A13" s="24" t="inlineStr">
         <is>
           <t>听力</t>
@@ -3628,7 +3628,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="21" customHeight="1">
+    <row r="14" ht="23" customHeight="1">
       <c r="A14" s="24" t="inlineStr">
         <is>
           <t>阅读</t>
@@ -3661,7 +3661,7 @@
       </c>
       <c r="G14" s="25" t="inlineStr"/>
     </row>
-    <row r="15" ht="21" customHeight="1">
+    <row r="15" ht="23" customHeight="1">
       <c r="A15" s="24" t="inlineStr">
         <is>
           <t>阅读</t>
@@ -3698,7 +3698,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="21" customHeight="1">
+    <row r="16" ht="23" customHeight="1">
       <c r="A16" s="24" t="inlineStr">
         <is>
           <t>阅读</t>
@@ -3735,7 +3735,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="21" customHeight="1">
+    <row r="17" ht="23" customHeight="1">
       <c r="A17" s="24" t="inlineStr">
         <is>
           <t>阅读</t>
@@ -3772,7 +3772,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="21" customHeight="1">
+    <row r="18" ht="23" customHeight="1">
       <c r="A18" s="24" t="inlineStr">
         <is>
           <t>阅读</t>
@@ -3809,7 +3809,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="21" customHeight="1">
+    <row r="19" ht="23" customHeight="1">
       <c r="A19" s="24" t="inlineStr">
         <is>
           <t>阅读</t>
@@ -3842,7 +3842,7 @@
       </c>
       <c r="G19" s="25" t="inlineStr"/>
     </row>
-    <row r="20" ht="21" customHeight="1">
+    <row r="20" ht="38" customHeight="1">
       <c r="A20" s="24" t="inlineStr">
         <is>
           <t>阅读</t>
@@ -3879,7 +3879,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="21" customHeight="1">
+    <row r="21" ht="38" customHeight="1">
       <c r="A21" s="24" t="inlineStr">
         <is>
           <t>阅读</t>
@@ -3916,7 +3916,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="21" customHeight="1">
+    <row r="22" ht="23" customHeight="1">
       <c r="A22" s="24" t="inlineStr">
         <is>
           <t>阅读</t>
@@ -3953,7 +3953,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="21" customHeight="1">
+    <row r="23" ht="38" customHeight="1">
       <c r="A23" s="24" t="inlineStr">
         <is>
           <t>阅读</t>
@@ -3990,7 +3990,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="21" customHeight="1">
+    <row r="24" ht="38" customHeight="1">
       <c r="A24" s="24" t="inlineStr">
         <is>
           <t>阅读</t>
@@ -4008,1136 +4008,1138 @@
       </c>
       <c r="D24" s="26" t="inlineStr">
         <is>
+          <t>choice</t>
+        </is>
+      </c>
+      <c r="E24" s="25" t="inlineStr">
+        <is>
+          <t>A~G 字母池，逐题选一个</t>
+        </is>
+      </c>
+      <c r="F24" s="25" t="inlineStr">
+        <is>
+          <t>3.0 L5、L7-9</t>
+        </is>
+      </c>
+      <c r="G24" s="25" t="inlineStr">
+        <is>
+          <t>实测答案均为单个字母（D/A/F/G），材料与字母池在 question_group → 单选；不做拖拽排序控件</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="23" customHeight="1">
+      <c r="A25" s="24" t="inlineStr">
+        <is>
+          <t>阅读</t>
+        </is>
+      </c>
+      <c r="B25" s="25" t="inlineStr">
+        <is>
+          <t>病句选择题</t>
+        </is>
+      </c>
+      <c r="C25" s="25" t="inlineStr">
+        <is>
+          <t>reading_wrong_sentence</t>
+        </is>
+      </c>
+      <c r="D25" s="26" t="inlineStr">
+        <is>
+          <t>choice</t>
+        </is>
+      </c>
+      <c r="E25" s="25" t="inlineStr">
+        <is>
+          <t>A~D 四个句子，选出病句</t>
+        </is>
+      </c>
+      <c r="F25" s="25" t="inlineStr">
+        <is>
+          <t>2.0 L6</t>
+        </is>
+      </c>
+      <c r="G25" s="25" t="inlineStr">
+        <is>
+          <t>3.0 已删除</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="23" customHeight="1">
+      <c r="A26" s="24" t="inlineStr">
+        <is>
+          <t>阅读</t>
+        </is>
+      </c>
+      <c r="B26" s="25" t="inlineStr">
+        <is>
+          <t>选词填空题</t>
+        </is>
+      </c>
+      <c r="C26" s="25" t="inlineStr">
+        <is>
+          <t>reading_word_fill</t>
+        </is>
+      </c>
+      <c r="D26" s="26" t="inlineStr">
+        <is>
+          <t>choice</t>
+        </is>
+      </c>
+      <c r="E26" s="25" t="inlineStr">
+        <is>
+          <t>每空 A~D 选词，单选</t>
+        </is>
+      </c>
+      <c r="F26" s="25" t="inlineStr">
+        <is>
+          <t>2.0 L6；3.0 L6</t>
+        </is>
+      </c>
+      <c r="G26" s="25" t="inlineStr"/>
+    </row>
+    <row r="27" ht="38" customHeight="1">
+      <c r="A27" s="24" t="inlineStr">
+        <is>
+          <t>阅读</t>
+        </is>
+      </c>
+      <c r="B27" s="25" t="inlineStr">
+        <is>
+          <t>文章简答题</t>
+        </is>
+      </c>
+      <c r="C27" s="25" t="inlineStr">
+        <is>
+          <t>reading_short_answer</t>
+        </is>
+      </c>
+      <c r="D27" s="26" t="inlineStr">
+        <is>
+          <t>input</t>
+        </is>
+      </c>
+      <c r="E27" s="25" t="inlineStr">
+        <is>
+          <t>多行文本框</t>
+        </is>
+      </c>
+      <c r="F27" s="25" t="inlineStr">
+        <is>
+          <t>3.0 L7-9</t>
+        </is>
+      </c>
+      <c r="G27" s="25" t="inlineStr">
+        <is>
+          <t>无选项，答案为一~两句话（最长 10 字），不适用单字输入框</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="38" customHeight="1">
+      <c r="A28" s="24" t="inlineStr">
+        <is>
+          <t>写作、书写</t>
+        </is>
+      </c>
+      <c r="B28" s="25" t="inlineStr">
+        <is>
+          <t>连词成句</t>
+        </is>
+      </c>
+      <c r="C28" s="25" t="inlineStr">
+        <is>
+          <t>writing_complete_sent</t>
+        </is>
+      </c>
+      <c r="D28" s="26" t="inlineStr">
+        <is>
           <t>order</t>
         </is>
       </c>
-      <c r="E24" s="25" t="inlineStr">
-        <is>
-          <t>A~E 五段排序，拖拽/填序列</t>
-        </is>
-      </c>
-      <c r="F24" s="25" t="inlineStr">
-        <is>
-          <t>3.0 L5、L7-9</t>
-        </is>
-      </c>
-      <c r="G24" s="25" t="inlineStr">
-        <is>
-          <t>段落文本在 question_group.passage</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="21" customHeight="1">
-      <c r="A25" s="24" t="inlineStr">
-        <is>
-          <t>阅读</t>
-        </is>
-      </c>
-      <c r="B25" s="25" t="inlineStr">
-        <is>
-          <t>病句选择题</t>
-        </is>
-      </c>
-      <c r="C25" s="25" t="inlineStr">
-        <is>
-          <t>reading_wrong_sentence</t>
-        </is>
-      </c>
-      <c r="D25" s="26" t="inlineStr">
+      <c r="E28" s="25" t="inlineStr">
+        <is>
+          <t>词块拖拽/点选排成句</t>
+        </is>
+      </c>
+      <c r="F28" s="25" t="inlineStr">
+        <is>
+          <t>2.0 L3–L5</t>
+        </is>
+      </c>
+      <c r="G28" s="25" t="inlineStr">
+        <is>
+          <t>打乱词序放在题面 passage，答案是整句（句末半角 .）</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="38" customHeight="1">
+      <c r="A29" s="24" t="inlineStr">
+        <is>
+          <t>写作、书写</t>
+        </is>
+      </c>
+      <c r="B29" s="25" t="inlineStr">
+        <is>
+          <t>汉字书写</t>
+        </is>
+      </c>
+      <c r="C29" s="25" t="inlineStr">
+        <is>
+          <t>writing_character</t>
+        </is>
+      </c>
+      <c r="D29" s="26" t="inlineStr">
+        <is>
+          <t>shortInput</t>
+        </is>
+      </c>
+      <c r="E29" s="25" t="inlineStr">
+        <is>
+          <t>单行输入框，maxlength=1</t>
+        </is>
+      </c>
+      <c r="F29" s="25" t="inlineStr">
+        <is>
+          <t>2.0 L3；3.0 L2、L3</t>
+        </is>
+      </c>
+      <c r="G29" s="25" t="inlineStr">
+        <is>
+          <t>答案恒为单个汉字；系统手写键盘输入，不自绘手写板</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="23" customHeight="1">
+      <c r="A30" s="24" t="inlineStr">
+        <is>
+          <t>写作、书写</t>
+        </is>
+      </c>
+      <c r="B30" s="25" t="inlineStr">
+        <is>
+          <t>汉字部件选择</t>
+        </is>
+      </c>
+      <c r="C30" s="25" t="inlineStr">
+        <is>
+          <t>writing_comp_choice</t>
+        </is>
+      </c>
+      <c r="D30" s="26" t="inlineStr">
         <is>
           <t>choice</t>
         </is>
       </c>
-      <c r="E25" s="25" t="inlineStr">
-        <is>
-          <t>A~D 四个句子，选出病句</t>
-        </is>
-      </c>
-      <c r="F25" s="25" t="inlineStr">
+      <c r="E30" s="25" t="inlineStr">
+        <is>
+          <t>A~D 部件选项，单选</t>
+        </is>
+      </c>
+      <c r="F30" s="25" t="inlineStr">
+        <is>
+          <t>3.0 L2</t>
+        </is>
+      </c>
+      <c r="G30" s="25" t="inlineStr">
+        <is>
+          <t>选部件不是写汉字，仍是选择题</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="23" customHeight="1">
+      <c r="A31" s="24" t="inlineStr">
+        <is>
+          <t>写作、书写</t>
+        </is>
+      </c>
+      <c r="B31" s="25" t="inlineStr">
+        <is>
+          <t>看图用词造句</t>
+        </is>
+      </c>
+      <c r="C31" s="25" t="inlineStr">
+        <is>
+          <t>writing_pic_sentence</t>
+        </is>
+      </c>
+      <c r="D31" s="26" t="inlineStr">
+        <is>
+          <t>input</t>
+        </is>
+      </c>
+      <c r="E31" s="25" t="inlineStr">
+        <is>
+          <t>单行/多行文本框</t>
+        </is>
+      </c>
+      <c r="F31" s="25" t="inlineStr">
+        <is>
+          <t>2.0 L4；3.0 L3、L4</t>
+        </is>
+      </c>
+      <c r="G31" s="25" t="inlineStr">
+        <is>
+          <t>写一句话，用给定词</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="23" customHeight="1">
+      <c r="A32" s="24" t="inlineStr">
+        <is>
+          <t>写作、书写</t>
+        </is>
+      </c>
+      <c r="B32" s="25" t="inlineStr">
+        <is>
+          <t>短文写作</t>
+        </is>
+      </c>
+      <c r="C32" s="25" t="inlineStr">
+        <is>
+          <t>writing_short_essay</t>
+        </is>
+      </c>
+      <c r="D32" s="26" t="inlineStr">
+        <is>
+          <t>input</t>
+        </is>
+      </c>
+      <c r="E32" s="25" t="inlineStr">
+        <is>
+          <t>多行文本框 + 字数提示</t>
+        </is>
+      </c>
+      <c r="F32" s="25" t="inlineStr">
+        <is>
+          <t>2.0 L5；3.0 L4</t>
+        </is>
+      </c>
+      <c r="G32" s="25" t="inlineStr"/>
+    </row>
+    <row r="33" ht="23" customHeight="1">
+      <c r="A33" s="24" t="inlineStr">
+        <is>
+          <t>写作、书写</t>
+        </is>
+      </c>
+      <c r="B33" s="25" t="inlineStr">
+        <is>
+          <t>看图写作</t>
+        </is>
+      </c>
+      <c r="C33" s="25" t="inlineStr">
+        <is>
+          <t>writing_pic_write</t>
+        </is>
+      </c>
+      <c r="D33" s="26" t="inlineStr">
+        <is>
+          <t>input</t>
+        </is>
+      </c>
+      <c r="E33" s="25" t="inlineStr">
+        <is>
+          <t>多行文本框 + 字数提示</t>
+        </is>
+      </c>
+      <c r="F33" s="25" t="inlineStr">
+        <is>
+          <t>3.0 L5</t>
+        </is>
+      </c>
+      <c r="G33" s="25" t="inlineStr"/>
+    </row>
+    <row r="34" ht="23" customHeight="1">
+      <c r="A34" s="24" t="inlineStr">
+        <is>
+          <t>写作、书写</t>
+        </is>
+      </c>
+      <c r="B34" s="25" t="inlineStr">
+        <is>
+          <t>话题作文</t>
+        </is>
+      </c>
+      <c r="C34" s="25" t="inlineStr">
+        <is>
+          <t>writing_topic_essay</t>
+        </is>
+      </c>
+      <c r="D34" s="26" t="inlineStr">
+        <is>
+          <t>input</t>
+        </is>
+      </c>
+      <c r="E34" s="25" t="inlineStr">
+        <is>
+          <t>多行文本框 + 字数提示</t>
+        </is>
+      </c>
+      <c r="F34" s="25" t="inlineStr">
+        <is>
+          <t>3.0 L5–L7-9</t>
+        </is>
+      </c>
+      <c r="G34" s="25" t="inlineStr">
+        <is>
+          <t>字数要求 ≥80 / ≥300 字，由题型决定提示</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="23" customHeight="1">
+      <c r="A35" s="24" t="inlineStr">
+        <is>
+          <t>写作、书写</t>
+        </is>
+      </c>
+      <c r="B35" s="25" t="inlineStr">
+        <is>
+          <t>应用文写作</t>
+        </is>
+      </c>
+      <c r="C35" s="25" t="inlineStr">
+        <is>
+          <t>writing_practical</t>
+        </is>
+      </c>
+      <c r="D35" s="26" t="inlineStr">
+        <is>
+          <t>input</t>
+        </is>
+      </c>
+      <c r="E35" s="25" t="inlineStr">
+        <is>
+          <t>多行文本框 + 字数提示</t>
+        </is>
+      </c>
+      <c r="F35" s="25" t="inlineStr">
+        <is>
+          <t>3.0 L6</t>
+        </is>
+      </c>
+      <c r="G35" s="25" t="inlineStr"/>
+    </row>
+    <row r="36" ht="23" customHeight="1">
+      <c r="A36" s="24" t="inlineStr">
+        <is>
+          <t>写作、书写</t>
+        </is>
+      </c>
+      <c r="B36" s="25" t="inlineStr">
+        <is>
+          <t>图表描述与分析</t>
+        </is>
+      </c>
+      <c r="C36" s="25" t="inlineStr">
+        <is>
+          <t>writing_chart_analysis</t>
+        </is>
+      </c>
+      <c r="D36" s="26" t="inlineStr">
+        <is>
+          <t>input</t>
+        </is>
+      </c>
+      <c r="E36" s="25" t="inlineStr">
+        <is>
+          <t>多行文本框 + 图表材料</t>
+        </is>
+      </c>
+      <c r="F36" s="25" t="inlineStr">
+        <is>
+          <t>3.0 L7-9</t>
+        </is>
+      </c>
+      <c r="G36" s="25" t="inlineStr">
+        <is>
+          <t>图表是材料不是选项，控件仍是文本框</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="23" customHeight="1">
+      <c r="A37" s="24" t="inlineStr">
+        <is>
+          <t>写作、书写</t>
+        </is>
+      </c>
+      <c r="B37" s="25" t="inlineStr">
+        <is>
+          <t>缩写作文</t>
+        </is>
+      </c>
+      <c r="C37" s="25" t="inlineStr">
+        <is>
+          <t>writing_summary</t>
+        </is>
+      </c>
+      <c r="D37" s="26" t="inlineStr">
+        <is>
+          <t>input</t>
+        </is>
+      </c>
+      <c r="E37" s="25" t="inlineStr">
+        <is>
+          <t>多行文本框 + 字数提示</t>
+        </is>
+      </c>
+      <c r="F37" s="25" t="inlineStr">
         <is>
           <t>2.0 L6</t>
         </is>
       </c>
-      <c r="G25" s="25" t="inlineStr">
-        <is>
-          <t>3.0 已删除</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="21" customHeight="1">
-      <c r="A26" s="24" t="inlineStr">
-        <is>
-          <t>阅读</t>
-        </is>
-      </c>
-      <c r="B26" s="25" t="inlineStr">
-        <is>
-          <t>选词填空题</t>
-        </is>
-      </c>
-      <c r="C26" s="25" t="inlineStr">
-        <is>
-          <t>reading_word_fill</t>
-        </is>
-      </c>
-      <c r="D26" s="26" t="inlineStr">
+      <c r="G37" s="25" t="inlineStr">
+        <is>
+          <t>答案字段为占位「略」，不作评分依据</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="23" customHeight="1">
+      <c r="A38" s="24" t="inlineStr">
+        <is>
+          <t>翻译</t>
+        </is>
+      </c>
+      <c r="B38" s="25" t="inlineStr">
+        <is>
+          <t>笔译</t>
+        </is>
+      </c>
+      <c r="C38" s="25" t="inlineStr">
+        <is>
+          <t>translation_written</t>
+        </is>
+      </c>
+      <c r="D38" s="26" t="inlineStr">
+        <is>
+          <t>input</t>
+        </is>
+      </c>
+      <c r="E38" s="25" t="inlineStr">
+        <is>
+          <t>多行文本框</t>
+        </is>
+      </c>
+      <c r="F38" s="25" t="inlineStr">
+        <is>
+          <t>3.0 L7-9</t>
+        </is>
+      </c>
+      <c r="G38" s="25" t="inlineStr"/>
+    </row>
+    <row r="39" ht="23" customHeight="1">
+      <c r="A39" s="24" t="inlineStr">
+        <is>
+          <t>翻译</t>
+        </is>
+      </c>
+      <c r="B39" s="25" t="inlineStr">
+        <is>
+          <t>口译</t>
+        </is>
+      </c>
+      <c r="C39" s="25" t="inlineStr">
+        <is>
+          <t>translation_oral</t>
+        </is>
+      </c>
+      <c r="D39" s="26" t="inlineStr">
+        <is>
+          <t>record</t>
+        </is>
+      </c>
+      <c r="E39" s="25" t="inlineStr">
+        <is>
+          <t>录音按钮 + 倒计时</t>
+        </is>
+      </c>
+      <c r="F39" s="25" t="inlineStr">
+        <is>
+          <t>3.0 L7-9</t>
+        </is>
+      </c>
+      <c r="G39" s="25" t="inlineStr">
+        <is>
+          <t>与口语同控件，仅题面换成外文原文</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="23" customHeight="1">
+      <c r="A40" s="24" t="inlineStr">
+        <is>
+          <t>口语</t>
+        </is>
+      </c>
+      <c r="B40" s="25" t="inlineStr">
+        <is>
+          <t>应用读说</t>
+        </is>
+      </c>
+      <c r="C40" s="25" t="inlineStr">
+        <is>
+          <t>speaking_read_aloud</t>
+        </is>
+      </c>
+      <c r="D40" s="26" t="inlineStr">
+        <is>
+          <t>record</t>
+        </is>
+      </c>
+      <c r="E40" s="25" t="inlineStr">
+        <is>
+          <t>录音按钮 + 倒计时</t>
+        </is>
+      </c>
+      <c r="F40" s="25" t="inlineStr">
+        <is>
+          <t>3.0 L7-9</t>
+        </is>
+      </c>
+      <c r="G40" s="25" t="inlineStr"/>
+    </row>
+    <row r="41" ht="23" customHeight="1">
+      <c r="A41" s="24" t="inlineStr">
+        <is>
+          <t>口语</t>
+        </is>
+      </c>
+      <c r="B41" s="25" t="inlineStr">
+        <is>
+          <t>听材料回答问题</t>
+        </is>
+      </c>
+      <c r="C41" s="25" t="inlineStr">
+        <is>
+          <t>speaking_listen_answer</t>
+        </is>
+      </c>
+      <c r="D41" s="26" t="inlineStr">
+        <is>
+          <t>record</t>
+        </is>
+      </c>
+      <c r="E41" s="25" t="inlineStr">
+        <is>
+          <t>录音按钮 + 倒计时</t>
+        </is>
+      </c>
+      <c r="F41" s="25" t="inlineStr">
+        <is>
+          <t>3.0 L7-9</t>
+        </is>
+      </c>
+      <c r="G41" s="25" t="inlineStr">
+        <is>
+          <t>与 HSKK「听后回答」不是同一题型，勿复用</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="23" customHeight="1">
+      <c r="A42" s="24" t="inlineStr">
+        <is>
+          <t>口语</t>
+        </is>
+      </c>
+      <c r="B42" s="25" t="inlineStr">
+        <is>
+          <t>观点表达</t>
+        </is>
+      </c>
+      <c r="C42" s="25" t="inlineStr">
+        <is>
+          <t>speaking_opinion</t>
+        </is>
+      </c>
+      <c r="D42" s="26" t="inlineStr">
+        <is>
+          <t>record</t>
+        </is>
+      </c>
+      <c r="E42" s="25" t="inlineStr">
+        <is>
+          <t>录音按钮 + 倒计时</t>
+        </is>
+      </c>
+      <c r="F42" s="25" t="inlineStr">
+        <is>
+          <t>3.0 L7-9</t>
+        </is>
+      </c>
+      <c r="G42" s="25" t="inlineStr"/>
+    </row>
+    <row r="43" ht="23" customHeight="1">
+      <c r="A43" s="24" t="inlineStr">
+        <is>
+          <t>HSKK 口语</t>
+        </is>
+      </c>
+      <c r="B43" s="25" t="inlineStr">
+        <is>
+          <t>听后重复</t>
+        </is>
+      </c>
+      <c r="C43" s="25" t="inlineStr">
+        <is>
+          <t>speaking_repeat</t>
+        </is>
+      </c>
+      <c r="D43" s="26" t="inlineStr">
+        <is>
+          <t>record</t>
+        </is>
+      </c>
+      <c r="E43" s="25" t="inlineStr">
+        <is>
+          <t>录音按钮 + 倒计时</t>
+        </is>
+      </c>
+      <c r="F43" s="25" t="inlineStr">
+        <is>
+          <t>2.0 初、中、高；3.0 L3</t>
+        </is>
+      </c>
+      <c r="G43" s="25" t="inlineStr">
+        <is>
+          <t>一句/一段后原样复述</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="23" customHeight="1">
+      <c r="A44" s="24" t="inlineStr">
+        <is>
+          <t>HSKK 口语</t>
+        </is>
+      </c>
+      <c r="B44" s="25" t="inlineStr">
+        <is>
+          <t>听后回答</t>
+        </is>
+      </c>
+      <c r="C44" s="25" t="inlineStr">
+        <is>
+          <t>speaking_listen_response</t>
+        </is>
+      </c>
+      <c r="D44" s="26" t="inlineStr">
+        <is>
+          <t>record</t>
+        </is>
+      </c>
+      <c r="E44" s="25" t="inlineStr">
+        <is>
+          <t>录音按钮 + 倒计时</t>
+        </is>
+      </c>
+      <c r="F44" s="25" t="inlineStr">
+        <is>
+          <t>2.0 初级</t>
+        </is>
+      </c>
+      <c r="G44" s="25" t="inlineStr">
+        <is>
+          <t>仅 HSKK2.0 初级第二部分</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="23" customHeight="1">
+      <c r="A45" s="24" t="inlineStr">
+        <is>
+          <t>HSKK 口语</t>
+        </is>
+      </c>
+      <c r="B45" s="25" t="inlineStr">
+        <is>
+          <t>听后复述</t>
+        </is>
+      </c>
+      <c r="C45" s="25" t="inlineStr">
+        <is>
+          <t>speaking_retell</t>
+        </is>
+      </c>
+      <c r="D45" s="26" t="inlineStr">
+        <is>
+          <t>record</t>
+        </is>
+      </c>
+      <c r="E45" s="25" t="inlineStr">
+        <is>
+          <t>录音按钮 + 倒计时</t>
+        </is>
+      </c>
+      <c r="F45" s="25" t="inlineStr">
+        <is>
+          <t>3.0 L4、L5、L6</t>
+        </is>
+      </c>
+      <c r="G45" s="25" t="inlineStr">
+        <is>
+          <t>3.0 四级起替代「听后重复」，材料更长</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="23" customHeight="1">
+      <c r="A46" s="24" t="inlineStr">
+        <is>
+          <t>HSKK 口语</t>
+        </is>
+      </c>
+      <c r="B46" s="25" t="inlineStr">
+        <is>
+          <t>看图说话</t>
+        </is>
+      </c>
+      <c r="C46" s="25" t="inlineStr">
+        <is>
+          <t>speaking_pic_describe</t>
+        </is>
+      </c>
+      <c r="D46" s="26" t="inlineStr">
+        <is>
+          <t>record</t>
+        </is>
+      </c>
+      <c r="E46" s="25" t="inlineStr">
+        <is>
+          <t>录音按钮 + 倒计时</t>
+        </is>
+      </c>
+      <c r="F46" s="25" t="inlineStr">
+        <is>
+          <t>2.0 中级；3.0 L3–L6</t>
+        </is>
+      </c>
+      <c r="G46" s="25" t="inlineStr">
+        <is>
+          <t>图是材料不是选项</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="38" customHeight="1">
+      <c r="A47" s="24" t="inlineStr">
+        <is>
+          <t>HSKK 口语</t>
+        </is>
+      </c>
+      <c r="B47" s="25" t="inlineStr">
+        <is>
+          <t>朗读</t>
+        </is>
+      </c>
+      <c r="C47" s="25" t="inlineStr">
+        <is>
+          <t>speaking_read_text</t>
+        </is>
+      </c>
+      <c r="D47" s="26" t="inlineStr">
+        <is>
+          <t>record</t>
+        </is>
+      </c>
+      <c r="E47" s="25" t="inlineStr">
+        <is>
+          <t>录音按钮 + 倒计时</t>
+        </is>
+      </c>
+      <c r="F47" s="25" t="inlineStr">
+        <is>
+          <t>2.0 高级</t>
+        </is>
+      </c>
+      <c r="G47" s="25" t="inlineStr">
+        <is>
+          <t>仅 HSKK2.0 高级第二部分；勿用 speaking_read_aloud</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="38" customHeight="1">
+      <c r="A48" s="24" t="inlineStr">
+        <is>
+          <t>HSKK 口语</t>
+        </is>
+      </c>
+      <c r="B48" s="25" t="inlineStr">
+        <is>
+          <t>回答问题</t>
+        </is>
+      </c>
+      <c r="C48" s="25" t="inlineStr">
+        <is>
+          <t>speaking_qa</t>
+        </is>
+      </c>
+      <c r="D48" s="26" t="inlineStr">
+        <is>
+          <t>record</t>
+        </is>
+      </c>
+      <c r="E48" s="25" t="inlineStr">
+        <is>
+          <t>录音按钮 + 倒计时</t>
+        </is>
+      </c>
+      <c r="F48" s="25" t="inlineStr">
+        <is>
+          <t>2.0 初、中、高；3.0 L3–L6</t>
+        </is>
+      </c>
+      <c r="G48" s="25" t="inlineStr">
+        <is>
+          <t>两版均有，恒 2 题/卷</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="8" customHeight="1"/>
+    <row r="50" ht="8" customHeight="1"/>
+    <row r="51" ht="28" customHeight="1">
+      <c r="A51" s="22" t="inlineStr">
+        <is>
+          <t>布局值清单（8 个，全库唯一合法取值）</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="38" customHeight="1">
+      <c r="A52" s="23" t="inlineStr">
+        <is>
+          <t>布局（layout）</t>
+        </is>
+      </c>
+      <c r="B52" s="23" t="inlineStr">
+        <is>
+          <t>含义</t>
+        </is>
+      </c>
+      <c r="C52" s="29" t="n"/>
+      <c r="D52" s="23" t="inlineStr">
+        <is>
+          <t>控件形态</t>
+        </is>
+      </c>
+      <c r="E52" s="29" t="n"/>
+      <c r="F52" s="23" t="inlineStr">
+        <is>
+          <t>本表题型数</t>
+        </is>
+      </c>
+      <c r="G52" s="23" t="inlineStr">
+        <is>
+          <t>数据落点</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="38" customHeight="1">
+      <c r="A53" s="26" t="inlineStr">
         <is>
           <t>choice</t>
         </is>
       </c>
-      <c r="E26" s="25" t="inlineStr">
-        <is>
-          <t>每空 A~D 选词，单选</t>
-        </is>
-      </c>
-      <c r="F26" s="25" t="inlineStr">
-        <is>
-          <t>2.0 L6；3.0 L6</t>
-        </is>
-      </c>
-      <c r="G26" s="25" t="inlineStr"/>
-    </row>
-    <row r="27" ht="36" customHeight="1">
-      <c r="A27" s="24" t="inlineStr">
-        <is>
-          <t>阅读</t>
-        </is>
-      </c>
-      <c r="B27" s="25" t="inlineStr">
-        <is>
-          <t>文章简答题</t>
-        </is>
-      </c>
-      <c r="C27" s="25" t="inlineStr">
-        <is>
-          <t>reading_short_answer</t>
-        </is>
-      </c>
-      <c r="D27" s="26" t="inlineStr">
+      <c r="B53" s="25" t="inlineStr">
+        <is>
+          <t>单选：一组选项选出一个</t>
+        </is>
+      </c>
+      <c r="C53" s="27" t="n"/>
+      <c r="D53" s="25" t="inlineStr">
+        <is>
+          <t>选项组 / 单选按钮</t>
+        </is>
+      </c>
+      <c r="E53" s="27" t="n"/>
+      <c r="F53" s="28" t="n">
+        <v>17</v>
+      </c>
+      <c r="G53" s="25" t="inlineStr">
+        <is>
+          <t>本题 option_content；分组共用时取组 option_content 池</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="38" customHeight="1">
+      <c r="A54" s="26" t="inlineStr">
+        <is>
+          <t>choiceGrid</t>
+        </is>
+      </c>
+      <c r="B54" s="25" t="inlineStr">
+        <is>
+          <t>网格匹配：同组共用一套选项池，逐题取一、选中置灰</t>
+        </is>
+      </c>
+      <c r="C54" s="27" t="n"/>
+      <c r="D54" s="25" t="inlineStr">
+        <is>
+          <t>A~E 网格格子（图或句）</t>
+        </is>
+      </c>
+      <c r="E54" s="27" t="n"/>
+      <c r="F54" s="28" t="n">
+        <v>2</v>
+      </c>
+      <c r="G54" s="25" t="inlineStr">
+        <is>
+          <t>分组 option_content 池</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="23" customHeight="1">
+      <c r="A55" s="26" t="inlineStr">
+        <is>
+          <t>judge</t>
+        </is>
+      </c>
+      <c r="B55" s="25" t="inlineStr">
+        <is>
+          <t>判断：二值 √/× 或三值 √/×/◯</t>
+        </is>
+      </c>
+      <c r="C55" s="27" t="n"/>
+      <c r="D55" s="25" t="inlineStr">
+        <is>
+          <t>判断按钮组</t>
+        </is>
+      </c>
+      <c r="E55" s="27" t="n"/>
+      <c r="F55" s="28" t="n">
+        <v>5</v>
+      </c>
+      <c r="G55" s="25" t="inlineStr">
+        <is>
+          <t>本题 option_content（A/B/C）</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="23" customHeight="1">
+      <c r="A56" s="26" t="inlineStr">
+        <is>
+          <t>multiChoice</t>
+        </is>
+      </c>
+      <c r="B56" s="25" t="inlineStr">
+        <is>
+          <t>多选：一个题干多个正确选项</t>
+        </is>
+      </c>
+      <c r="C56" s="27" t="n"/>
+      <c r="D56" s="25" t="inlineStr">
+        <is>
+          <t>复选按钮组</t>
+        </is>
+      </c>
+      <c r="E56" s="27" t="n"/>
+      <c r="F56" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="G56" s="25" t="inlineStr">
+        <is>
+          <t>本题 option_content；答案含逗号</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="23" customHeight="1">
+      <c r="A57" s="26" t="inlineStr">
+        <is>
+          <t>order</t>
+        </is>
+      </c>
+      <c r="B57" s="25" t="inlineStr">
+        <is>
+          <t>排序：词块成句 / 句子成段</t>
+        </is>
+      </c>
+      <c r="C57" s="27" t="n"/>
+      <c r="D57" s="25" t="inlineStr">
+        <is>
+          <t>拖拽排序或填字母序列</t>
+        </is>
+      </c>
+      <c r="E57" s="27" t="n"/>
+      <c r="F57" s="28" t="n">
+        <v>2</v>
+      </c>
+      <c r="G57" s="25" t="inlineStr">
+        <is>
+          <t>题面 passage 放打乱的材料，答案存字母序列或整句</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="23" customHeight="1">
+      <c r="A58" s="26" t="inlineStr">
         <is>
           <t>input</t>
         </is>
       </c>
-      <c r="E27" s="25" t="inlineStr">
-        <is>
-          <t>多行文本框</t>
-        </is>
-      </c>
-      <c r="F27" s="25" t="inlineStr">
-        <is>
-          <t>3.0 L7-9</t>
-        </is>
-      </c>
-      <c r="G27" s="25" t="inlineStr">
-        <is>
-          <t>无选项，答案为一~两句话（最长 10 字），不适用单字输入框</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="21" customHeight="1">
-      <c r="A28" s="24" t="inlineStr">
-        <is>
-          <t>写作、书写</t>
-        </is>
-      </c>
-      <c r="B28" s="25" t="inlineStr">
-        <is>
-          <t>连词成句</t>
-        </is>
-      </c>
-      <c r="C28" s="25" t="inlineStr">
-        <is>
-          <t>writing_complete_sent</t>
-        </is>
-      </c>
-      <c r="D28" s="26" t="inlineStr">
-        <is>
-          <t>order</t>
-        </is>
-      </c>
-      <c r="E28" s="25" t="inlineStr">
-        <is>
-          <t>词块拖拽/点选排成句</t>
-        </is>
-      </c>
-      <c r="F28" s="25" t="inlineStr">
-        <is>
-          <t>2.0 L3–L5</t>
-        </is>
-      </c>
-      <c r="G28" s="25" t="inlineStr">
-        <is>
-          <t>打乱词序放在题面 passage，答案是整句（句末半角 .）</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="21" customHeight="1">
-      <c r="A29" s="24" t="inlineStr">
-        <is>
-          <t>写作、书写</t>
-        </is>
-      </c>
-      <c r="B29" s="25" t="inlineStr">
-        <is>
-          <t>汉字书写</t>
-        </is>
-      </c>
-      <c r="C29" s="25" t="inlineStr">
-        <is>
-          <t>writing_character</t>
-        </is>
-      </c>
-      <c r="D29" s="26" t="inlineStr">
+      <c r="B58" s="25" t="inlineStr">
+        <is>
+          <t>文本输入：句子 / 短文 / 短答</t>
+        </is>
+      </c>
+      <c r="C58" s="27" t="n"/>
+      <c r="D58" s="25" t="inlineStr">
+        <is>
+          <t>多行文本框（按题型给字数提示）</t>
+        </is>
+      </c>
+      <c r="E58" s="27" t="n"/>
+      <c r="F58" s="28" t="n">
+        <v>9</v>
+      </c>
+      <c r="G58" s="25" t="inlineStr">
+        <is>
+          <t>作答文本</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="23" customHeight="1">
+      <c r="A59" s="26" t="inlineStr">
         <is>
           <t>shortInput</t>
         </is>
       </c>
-      <c r="E29" s="25" t="inlineStr">
+      <c r="B59" s="25" t="inlineStr">
+        <is>
+          <t>短文本输入：答案恒为单个汉字</t>
+        </is>
+      </c>
+      <c r="C59" s="27" t="n"/>
+      <c r="D59" s="25" t="inlineStr">
         <is>
           <t>单行输入框，maxlength=1</t>
         </is>
       </c>
-      <c r="F29" s="25" t="inlineStr">
-        <is>
-          <t>2.0 L3；3.0 L2、L3</t>
-        </is>
-      </c>
-      <c r="G29" s="25" t="inlineStr">
-        <is>
-          <t>答案恒为单个汉字；系统手写键盘输入，不自绘手写板</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="21" customHeight="1">
-      <c r="A30" s="24" t="inlineStr">
-        <is>
-          <t>写作、书写</t>
-        </is>
-      </c>
-      <c r="B30" s="25" t="inlineStr">
-        <is>
-          <t>汉字部件选择</t>
-        </is>
-      </c>
-      <c r="C30" s="25" t="inlineStr">
-        <is>
-          <t>writing_comp_choice</t>
-        </is>
-      </c>
-      <c r="D30" s="26" t="inlineStr">
-        <is>
-          <t>choice</t>
-        </is>
-      </c>
-      <c r="E30" s="25" t="inlineStr">
-        <is>
-          <t>A~D 部件选项，单选</t>
-        </is>
-      </c>
-      <c r="F30" s="25" t="inlineStr">
-        <is>
-          <t>3.0 L2</t>
-        </is>
-      </c>
-      <c r="G30" s="25" t="inlineStr">
-        <is>
-          <t>选部件不是写汉字，仍是选择题</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="21" customHeight="1">
-      <c r="A31" s="24" t="inlineStr">
-        <is>
-          <t>写作、书写</t>
-        </is>
-      </c>
-      <c r="B31" s="25" t="inlineStr">
-        <is>
-          <t>看图用词造句</t>
-        </is>
-      </c>
-      <c r="C31" s="25" t="inlineStr">
-        <is>
-          <t>writing_pic_sentence</t>
-        </is>
-      </c>
-      <c r="D31" s="26" t="inlineStr">
-        <is>
-          <t>input</t>
-        </is>
-      </c>
-      <c r="E31" s="25" t="inlineStr">
-        <is>
-          <t>单行/多行文本框</t>
-        </is>
-      </c>
-      <c r="F31" s="25" t="inlineStr">
-        <is>
-          <t>2.0 L4；3.0 L3、L4</t>
-        </is>
-      </c>
-      <c r="G31" s="25" t="inlineStr">
-        <is>
-          <t>写一句话，用给定词</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="21" customHeight="1">
-      <c r="A32" s="24" t="inlineStr">
-        <is>
-          <t>写作、书写</t>
-        </is>
-      </c>
-      <c r="B32" s="25" t="inlineStr">
-        <is>
-          <t>短文写作</t>
-        </is>
-      </c>
-      <c r="C32" s="25" t="inlineStr">
-        <is>
-          <t>writing_short_essay</t>
-        </is>
-      </c>
-      <c r="D32" s="26" t="inlineStr">
-        <is>
-          <t>input</t>
-        </is>
-      </c>
-      <c r="E32" s="25" t="inlineStr">
-        <is>
-          <t>多行文本框 + 字数提示</t>
-        </is>
-      </c>
-      <c r="F32" s="25" t="inlineStr">
-        <is>
-          <t>2.0 L5；3.0 L4</t>
-        </is>
-      </c>
-      <c r="G32" s="25" t="inlineStr"/>
-    </row>
-    <row r="33" ht="21" customHeight="1">
-      <c r="A33" s="24" t="inlineStr">
-        <is>
-          <t>写作、书写</t>
-        </is>
-      </c>
-      <c r="B33" s="25" t="inlineStr">
-        <is>
-          <t>看图写作</t>
-        </is>
-      </c>
-      <c r="C33" s="25" t="inlineStr">
-        <is>
-          <t>writing_pic_write</t>
-        </is>
-      </c>
-      <c r="D33" s="26" t="inlineStr">
-        <is>
-          <t>input</t>
-        </is>
-      </c>
-      <c r="E33" s="25" t="inlineStr">
-        <is>
-          <t>多行文本框 + 字数提示</t>
-        </is>
-      </c>
-      <c r="F33" s="25" t="inlineStr">
-        <is>
-          <t>3.0 L5</t>
-        </is>
-      </c>
-      <c r="G33" s="25" t="inlineStr"/>
-    </row>
-    <row r="34" ht="21" customHeight="1">
-      <c r="A34" s="24" t="inlineStr">
-        <is>
-          <t>写作、书写</t>
-        </is>
-      </c>
-      <c r="B34" s="25" t="inlineStr">
-        <is>
-          <t>话题作文</t>
-        </is>
-      </c>
-      <c r="C34" s="25" t="inlineStr">
-        <is>
-          <t>writing_topic_essay</t>
-        </is>
-      </c>
-      <c r="D34" s="26" t="inlineStr">
-        <is>
-          <t>input</t>
-        </is>
-      </c>
-      <c r="E34" s="25" t="inlineStr">
-        <is>
-          <t>多行文本框 + 字数提示</t>
-        </is>
-      </c>
-      <c r="F34" s="25" t="inlineStr">
-        <is>
-          <t>3.0 L5–L7-9</t>
-        </is>
-      </c>
-      <c r="G34" s="25" t="inlineStr">
-        <is>
-          <t>字数要求 ≥80 / ≥300 字，由题型决定提示</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="21" customHeight="1">
-      <c r="A35" s="24" t="inlineStr">
-        <is>
-          <t>写作、书写</t>
-        </is>
-      </c>
-      <c r="B35" s="25" t="inlineStr">
-        <is>
-          <t>应用文写作</t>
-        </is>
-      </c>
-      <c r="C35" s="25" t="inlineStr">
-        <is>
-          <t>writing_practical</t>
-        </is>
-      </c>
-      <c r="D35" s="26" t="inlineStr">
-        <is>
-          <t>input</t>
-        </is>
-      </c>
-      <c r="E35" s="25" t="inlineStr">
-        <is>
-          <t>多行文本框 + 字数提示</t>
-        </is>
-      </c>
-      <c r="F35" s="25" t="inlineStr">
-        <is>
-          <t>3.0 L6</t>
-        </is>
-      </c>
-      <c r="G35" s="25" t="inlineStr"/>
-    </row>
-    <row r="36" ht="21" customHeight="1">
-      <c r="A36" s="24" t="inlineStr">
-        <is>
-          <t>写作、书写</t>
-        </is>
-      </c>
-      <c r="B36" s="25" t="inlineStr">
-        <is>
-          <t>图表描述与分析</t>
-        </is>
-      </c>
-      <c r="C36" s="25" t="inlineStr">
-        <is>
-          <t>writing_chart_analysis</t>
-        </is>
-      </c>
-      <c r="D36" s="26" t="inlineStr">
-        <is>
-          <t>input</t>
-        </is>
-      </c>
-      <c r="E36" s="25" t="inlineStr">
-        <is>
-          <t>多行文本框 + 图表材料</t>
-        </is>
-      </c>
-      <c r="F36" s="25" t="inlineStr">
-        <is>
-          <t>3.0 L7-9</t>
-        </is>
-      </c>
-      <c r="G36" s="25" t="inlineStr">
-        <is>
-          <t>图表是材料不是选项，控件仍是文本框</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="21" customHeight="1">
-      <c r="A37" s="24" t="inlineStr">
-        <is>
-          <t>写作、书写</t>
-        </is>
-      </c>
-      <c r="B37" s="25" t="inlineStr">
-        <is>
-          <t>缩写作文</t>
-        </is>
-      </c>
-      <c r="C37" s="25" t="inlineStr">
-        <is>
-          <t>writing_summary</t>
-        </is>
-      </c>
-      <c r="D37" s="26" t="inlineStr">
-        <is>
-          <t>input</t>
-        </is>
-      </c>
-      <c r="E37" s="25" t="inlineStr">
-        <is>
-          <t>多行文本框 + 字数提示</t>
-        </is>
-      </c>
-      <c r="F37" s="25" t="inlineStr">
-        <is>
-          <t>2.0 L6</t>
-        </is>
-      </c>
-      <c r="G37" s="25" t="inlineStr">
-        <is>
-          <t>答案字段为占位「略」，不作评分依据</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="21" customHeight="1">
-      <c r="A38" s="24" t="inlineStr">
-        <is>
-          <t>翻译</t>
-        </is>
-      </c>
-      <c r="B38" s="25" t="inlineStr">
-        <is>
-          <t>笔译</t>
-        </is>
-      </c>
-      <c r="C38" s="25" t="inlineStr">
-        <is>
-          <t>translation_written</t>
-        </is>
-      </c>
-      <c r="D38" s="26" t="inlineStr">
-        <is>
-          <t>input</t>
-        </is>
-      </c>
-      <c r="E38" s="25" t="inlineStr">
-        <is>
-          <t>多行文本框</t>
-        </is>
-      </c>
-      <c r="F38" s="25" t="inlineStr">
-        <is>
-          <t>3.0 L7-9</t>
-        </is>
-      </c>
-      <c r="G38" s="25" t="inlineStr"/>
-    </row>
-    <row r="39" ht="21" customHeight="1">
-      <c r="A39" s="24" t="inlineStr">
-        <is>
-          <t>翻译</t>
-        </is>
-      </c>
-      <c r="B39" s="25" t="inlineStr">
-        <is>
-          <t>口译</t>
-        </is>
-      </c>
-      <c r="C39" s="25" t="inlineStr">
-        <is>
-          <t>translation_oral</t>
-        </is>
-      </c>
-      <c r="D39" s="26" t="inlineStr">
+      <c r="E59" s="27" t="n"/>
+      <c r="F59" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="G59" s="25" t="inlineStr">
+        <is>
+          <t>作答文本（1 个字符）</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="23" customHeight="1">
+      <c r="A60" s="26" t="inlineStr">
         <is>
           <t>record</t>
         </is>
       </c>
-      <c r="E39" s="25" t="inlineStr">
-        <is>
-          <t>录音按钮 + 倒计时</t>
-        </is>
-      </c>
-      <c r="F39" s="25" t="inlineStr">
-        <is>
-          <t>3.0 L7-9</t>
-        </is>
-      </c>
-      <c r="G39" s="25" t="inlineStr">
-        <is>
-          <t>与口语同控件，仅题面换成外文原文</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="21" customHeight="1">
-      <c r="A40" s="24" t="inlineStr">
-        <is>
-          <t>口语</t>
-        </is>
-      </c>
-      <c r="B40" s="25" t="inlineStr">
-        <is>
-          <t>应用读说</t>
-        </is>
-      </c>
-      <c r="C40" s="25" t="inlineStr">
-        <is>
-          <t>speaking_read_aloud</t>
-        </is>
-      </c>
-      <c r="D40" s="26" t="inlineStr">
-        <is>
-          <t>record</t>
-        </is>
-      </c>
-      <c r="E40" s="25" t="inlineStr">
-        <is>
-          <t>录音按钮 + 倒计时</t>
-        </is>
-      </c>
-      <c r="F40" s="25" t="inlineStr">
-        <is>
-          <t>3.0 L7-9</t>
-        </is>
-      </c>
-      <c r="G40" s="25" t="inlineStr"/>
-    </row>
-    <row r="41" ht="21" customHeight="1">
-      <c r="A41" s="24" t="inlineStr">
-        <is>
-          <t>口语</t>
-        </is>
-      </c>
-      <c r="B41" s="25" t="inlineStr">
-        <is>
-          <t>听材料回答问题</t>
-        </is>
-      </c>
-      <c r="C41" s="25" t="inlineStr">
-        <is>
-          <t>speaking_listen_answer</t>
-        </is>
-      </c>
-      <c r="D41" s="26" t="inlineStr">
-        <is>
-          <t>record</t>
-        </is>
-      </c>
-      <c r="E41" s="25" t="inlineStr">
-        <is>
-          <t>录音按钮 + 倒计时</t>
-        </is>
-      </c>
-      <c r="F41" s="25" t="inlineStr">
-        <is>
-          <t>3.0 L7-9</t>
-        </is>
-      </c>
-      <c r="G41" s="25" t="inlineStr">
-        <is>
-          <t>与 HSKK「听后回答」不是同一题型，勿复用</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="21" customHeight="1">
-      <c r="A42" s="24" t="inlineStr">
-        <is>
-          <t>口语</t>
-        </is>
-      </c>
-      <c r="B42" s="25" t="inlineStr">
-        <is>
-          <t>观点表达</t>
-        </is>
-      </c>
-      <c r="C42" s="25" t="inlineStr">
-        <is>
-          <t>speaking_opinion</t>
-        </is>
-      </c>
-      <c r="D42" s="26" t="inlineStr">
-        <is>
-          <t>record</t>
-        </is>
-      </c>
-      <c r="E42" s="25" t="inlineStr">
-        <is>
-          <t>录音按钮 + 倒计时</t>
-        </is>
-      </c>
-      <c r="F42" s="25" t="inlineStr">
-        <is>
-          <t>3.0 L7-9</t>
-        </is>
-      </c>
-      <c r="G42" s="25" t="inlineStr"/>
-    </row>
-    <row r="43" ht="21" customHeight="1">
-      <c r="A43" s="24" t="inlineStr">
-        <is>
-          <t>HSKK 口语</t>
-        </is>
-      </c>
-      <c r="B43" s="25" t="inlineStr">
-        <is>
-          <t>听后重复</t>
-        </is>
-      </c>
-      <c r="C43" s="25" t="inlineStr">
-        <is>
-          <t>speaking_repeat</t>
-        </is>
-      </c>
-      <c r="D43" s="26" t="inlineStr">
-        <is>
-          <t>record</t>
-        </is>
-      </c>
-      <c r="E43" s="25" t="inlineStr">
-        <is>
-          <t>录音按钮 + 倒计时</t>
-        </is>
-      </c>
-      <c r="F43" s="25" t="inlineStr">
-        <is>
-          <t>2.0 初、中、高；3.0 L3</t>
-        </is>
-      </c>
-      <c r="G43" s="25" t="inlineStr">
-        <is>
-          <t>一句/一段后原样复述</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="21" customHeight="1">
-      <c r="A44" s="24" t="inlineStr">
-        <is>
-          <t>HSKK 口语</t>
-        </is>
-      </c>
-      <c r="B44" s="25" t="inlineStr">
-        <is>
-          <t>听后回答</t>
-        </is>
-      </c>
-      <c r="C44" s="25" t="inlineStr">
-        <is>
-          <t>speaking_listen_response</t>
-        </is>
-      </c>
-      <c r="D44" s="26" t="inlineStr">
-        <is>
-          <t>record</t>
-        </is>
-      </c>
-      <c r="E44" s="25" t="inlineStr">
-        <is>
-          <t>录音按钮 + 倒计时</t>
-        </is>
-      </c>
-      <c r="F44" s="25" t="inlineStr">
-        <is>
-          <t>2.0 初级</t>
-        </is>
-      </c>
-      <c r="G44" s="25" t="inlineStr">
-        <is>
-          <t>仅 HSKK2.0 初级第二部分</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="21" customHeight="1">
-      <c r="A45" s="24" t="inlineStr">
-        <is>
-          <t>HSKK 口语</t>
-        </is>
-      </c>
-      <c r="B45" s="25" t="inlineStr">
-        <is>
-          <t>听后复述</t>
-        </is>
-      </c>
-      <c r="C45" s="25" t="inlineStr">
-        <is>
-          <t>speaking_retell</t>
-        </is>
-      </c>
-      <c r="D45" s="26" t="inlineStr">
-        <is>
-          <t>record</t>
-        </is>
-      </c>
-      <c r="E45" s="25" t="inlineStr">
-        <is>
-          <t>录音按钮 + 倒计时</t>
-        </is>
-      </c>
-      <c r="F45" s="25" t="inlineStr">
-        <is>
-          <t>3.0 L4、L5、L6</t>
-        </is>
-      </c>
-      <c r="G45" s="25" t="inlineStr">
-        <is>
-          <t>3.0 四级起替代「听后重复」，材料更长</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" ht="21" customHeight="1">
-      <c r="A46" s="24" t="inlineStr">
-        <is>
-          <t>HSKK 口语</t>
-        </is>
-      </c>
-      <c r="B46" s="25" t="inlineStr">
-        <is>
-          <t>看图说话</t>
-        </is>
-      </c>
-      <c r="C46" s="25" t="inlineStr">
-        <is>
-          <t>speaking_pic_describe</t>
-        </is>
-      </c>
-      <c r="D46" s="26" t="inlineStr">
-        <is>
-          <t>record</t>
-        </is>
-      </c>
-      <c r="E46" s="25" t="inlineStr">
-        <is>
-          <t>录音按钮 + 倒计时</t>
-        </is>
-      </c>
-      <c r="F46" s="25" t="inlineStr">
-        <is>
-          <t>2.0 中级；3.0 L3–L6</t>
-        </is>
-      </c>
-      <c r="G46" s="25" t="inlineStr">
-        <is>
-          <t>图是材料不是选项</t>
-        </is>
-      </c>
-    </row>
-    <row r="47" ht="21" customHeight="1">
-      <c r="A47" s="24" t="inlineStr">
-        <is>
-          <t>HSKK 口语</t>
-        </is>
-      </c>
-      <c r="B47" s="25" t="inlineStr">
-        <is>
-          <t>朗读</t>
-        </is>
-      </c>
-      <c r="C47" s="25" t="inlineStr">
-        <is>
-          <t>speaking_read_text</t>
-        </is>
-      </c>
-      <c r="D47" s="26" t="inlineStr">
-        <is>
-          <t>record</t>
-        </is>
-      </c>
-      <c r="E47" s="25" t="inlineStr">
-        <is>
-          <t>录音按钮 + 倒计时</t>
-        </is>
-      </c>
-      <c r="F47" s="25" t="inlineStr">
-        <is>
-          <t>2.0 高级</t>
-        </is>
-      </c>
-      <c r="G47" s="25" t="inlineStr">
-        <is>
-          <t>仅 HSKK2.0 高级第二部分；勿用 speaking_read_aloud</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="21" customHeight="1">
-      <c r="A48" s="24" t="inlineStr">
-        <is>
-          <t>HSKK 口语</t>
-        </is>
-      </c>
-      <c r="B48" s="25" t="inlineStr">
-        <is>
-          <t>回答问题</t>
-        </is>
-      </c>
-      <c r="C48" s="25" t="inlineStr">
-        <is>
-          <t>speaking_qa</t>
-        </is>
-      </c>
-      <c r="D48" s="26" t="inlineStr">
-        <is>
-          <t>record</t>
-        </is>
-      </c>
-      <c r="E48" s="25" t="inlineStr">
-        <is>
-          <t>录音按钮 + 倒计时</t>
-        </is>
-      </c>
-      <c r="F48" s="25" t="inlineStr">
-        <is>
-          <t>2.0 初、中、高；3.0 L3–L6</t>
-        </is>
-      </c>
-      <c r="G48" s="25" t="inlineStr">
-        <is>
-          <t>两版均有，恒 2 题/卷</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="26" customHeight="1">
-      <c r="A51" s="22" t="inlineStr">
-        <is>
-          <t>布局值清单（8 个，全库唯一合法取值）</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" ht="26" customHeight="1">
-      <c r="A52" s="23" t="inlineStr">
-        <is>
-          <t>布局（layout）</t>
-        </is>
-      </c>
-      <c r="B52" s="23" t="inlineStr">
-        <is>
-          <t>含义</t>
-        </is>
-      </c>
-      <c r="C52" s="23" t="inlineStr">
-        <is>
-          <t>控件形态</t>
-        </is>
-      </c>
-      <c r="D52" s="23" t="inlineStr">
-        <is>
-          <t>数据落点</t>
-        </is>
-      </c>
-      <c r="E52" s="23" t="inlineStr">
-        <is>
-          <t>本表题型数</t>
-        </is>
-      </c>
-      <c r="F52" s="27" t="n"/>
-      <c r="G52" s="27" t="n"/>
-    </row>
-    <row r="53" ht="66" customHeight="1">
-      <c r="A53" s="26" t="inlineStr">
-        <is>
-          <t>choice</t>
-        </is>
-      </c>
-      <c r="B53" s="25" t="inlineStr">
-        <is>
-          <t>单选：一组选项选出一个</t>
-        </is>
-      </c>
-      <c r="C53" s="25" t="inlineStr">
-        <is>
-          <t>选项组 / 单选按钮</t>
-        </is>
-      </c>
-      <c r="D53" s="25" t="inlineStr">
-        <is>
-          <t>本题 option_content；分组共用时取组 option_content 池</t>
-        </is>
-      </c>
-      <c r="E53" s="28" t="n">
-        <v>16</v>
-      </c>
-      <c r="F53" s="27" t="n"/>
-      <c r="G53" s="27" t="n"/>
-    </row>
-    <row r="54" ht="51" customHeight="1">
-      <c r="A54" s="26" t="inlineStr">
-        <is>
-          <t>choiceGrid</t>
-        </is>
-      </c>
-      <c r="B54" s="25" t="inlineStr">
-        <is>
-          <t>网格匹配：同组共用一套选项池，逐题取一、选中置灰</t>
-        </is>
-      </c>
-      <c r="C54" s="25" t="inlineStr">
-        <is>
-          <t>A~E 网格格子（图或句）</t>
-        </is>
-      </c>
-      <c r="D54" s="25" t="inlineStr">
-        <is>
-          <t>分组 option_content 池</t>
-        </is>
-      </c>
-      <c r="E54" s="28" t="n">
-        <v>2</v>
-      </c>
-      <c r="F54" s="27" t="n"/>
-      <c r="G54" s="27" t="n"/>
-    </row>
-    <row r="55" ht="51" customHeight="1">
-      <c r="A55" s="26" t="inlineStr">
-        <is>
-          <t>judge</t>
-        </is>
-      </c>
-      <c r="B55" s="25" t="inlineStr">
-        <is>
-          <t>判断：二值 √/× 或三值 √/×/◯</t>
-        </is>
-      </c>
-      <c r="C55" s="25" t="inlineStr">
-        <is>
-          <t>判断按钮组</t>
-        </is>
-      </c>
-      <c r="D55" s="25" t="inlineStr">
-        <is>
-          <t>本题 option_content（A/B/C）</t>
-        </is>
-      </c>
-      <c r="E55" s="28" t="n">
-        <v>5</v>
-      </c>
-      <c r="F55" s="27" t="n"/>
-      <c r="G55" s="27" t="n"/>
-    </row>
-    <row r="56" ht="51" customHeight="1">
-      <c r="A56" s="26" t="inlineStr">
-        <is>
-          <t>multiChoice</t>
-        </is>
-      </c>
-      <c r="B56" s="25" t="inlineStr">
-        <is>
-          <t>多选：一个题干多个正确选项</t>
-        </is>
-      </c>
-      <c r="C56" s="25" t="inlineStr">
-        <is>
-          <t>复选按钮组</t>
-        </is>
-      </c>
-      <c r="D56" s="25" t="inlineStr">
-        <is>
-          <t>本题 option_content；答案含逗号</t>
-        </is>
-      </c>
-      <c r="E56" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="F56" s="27" t="n"/>
-      <c r="G56" s="27" t="n"/>
-    </row>
-    <row r="57" ht="66" customHeight="1">
-      <c r="A57" s="26" t="inlineStr">
-        <is>
-          <t>order</t>
-        </is>
-      </c>
-      <c r="B57" s="25" t="inlineStr">
-        <is>
-          <t>排序：词块成句 / 句子成段</t>
-        </is>
-      </c>
-      <c r="C57" s="25" t="inlineStr">
-        <is>
-          <t>拖拽排序或填字母序列</t>
-        </is>
-      </c>
-      <c r="D57" s="25" t="inlineStr">
-        <is>
-          <t>题面 passage 放打乱的材料，答案存字母序列或整句</t>
-        </is>
-      </c>
-      <c r="E57" s="28" t="n">
-        <v>3</v>
-      </c>
-      <c r="F57" s="27" t="n"/>
-      <c r="G57" s="27" t="n"/>
-    </row>
-    <row r="58" ht="36" customHeight="1">
-      <c r="A58" s="26" t="inlineStr">
-        <is>
-          <t>input</t>
-        </is>
-      </c>
-      <c r="B58" s="25" t="inlineStr">
-        <is>
-          <t>文本输入：句子 / 短文 / 短答</t>
-        </is>
-      </c>
-      <c r="C58" s="25" t="inlineStr">
-        <is>
-          <t>多行文本框（按题型给字数提示）</t>
-        </is>
-      </c>
-      <c r="D58" s="25" t="inlineStr">
-        <is>
-          <t>作答文本</t>
-        </is>
-      </c>
-      <c r="E58" s="28" t="n">
-        <v>9</v>
-      </c>
-      <c r="F58" s="27" t="n"/>
-      <c r="G58" s="27" t="n"/>
-    </row>
-    <row r="59" ht="36" customHeight="1">
-      <c r="A59" s="26" t="inlineStr">
-        <is>
-          <t>shortInput</t>
-        </is>
-      </c>
-      <c r="B59" s="25" t="inlineStr">
-        <is>
-          <t>短文本输入：答案恒为单个汉字</t>
-        </is>
-      </c>
-      <c r="C59" s="25" t="inlineStr">
-        <is>
-          <t>单行输入框，maxlength=1</t>
-        </is>
-      </c>
-      <c r="D59" s="25" t="inlineStr">
-        <is>
-          <t>作答文本（1 个字符）</t>
-        </is>
-      </c>
-      <c r="E59" s="28" t="n">
-        <v>1</v>
-      </c>
-      <c r="F59" s="27" t="n"/>
-      <c r="G59" s="27" t="n"/>
-    </row>
-    <row r="60" ht="36" customHeight="1">
-      <c r="A60" s="26" t="inlineStr">
-        <is>
-          <t>record</t>
-        </is>
-      </c>
       <c r="B60" s="25" t="inlineStr">
         <is>
           <t>录音：口语 / 口译</t>
         </is>
       </c>
-      <c r="C60" s="25" t="inlineStr">
+      <c r="C60" s="27" t="n"/>
+      <c r="D60" s="25" t="inlineStr">
         <is>
           <t>录音按钮 + 倒计时 + 试听</t>
         </is>
       </c>
-      <c r="D60" s="25" t="inlineStr">
+      <c r="E60" s="27" t="n"/>
+      <c r="F60" s="28" t="n">
+        <v>10</v>
+      </c>
+      <c r="G60" s="25" t="inlineStr">
         <is>
           <t>音频对象，落在答卷侧</t>
         </is>
       </c>
-      <c r="E60" s="28" t="n">
-        <v>10</v>
-      </c>
-      <c r="F60" s="27" t="n"/>
-      <c r="G60" s="27" t="n"/>
     </row>
     <row r="61" ht="24" customHeight="1">
       <c r="A61" s="23" t="inlineStr">
@@ -5148,22 +5150,22 @@
       <c r="B61" s="29" t="n"/>
       <c r="C61" s="29" t="n"/>
       <c r="D61" s="29" t="n"/>
-      <c r="E61" s="23" t="inlineStr">
-        <is>
-          <t>46 个题型</t>
-        </is>
-      </c>
-      <c r="F61" s="29" t="n"/>
+      <c r="E61" s="29" t="n"/>
+      <c r="F61" s="23" t="n">
+        <v>46</v>
+      </c>
       <c r="G61" s="29" t="n"/>
     </row>
-    <row r="64" ht="26" customHeight="1">
+    <row r="62" ht="8" customHeight="1"/>
+    <row r="63" ht="8" customHeight="1"/>
+    <row r="64" ht="28" customHeight="1">
       <c r="A64" s="22" t="inlineStr">
         <is>
           <t>判定规则</t>
         </is>
       </c>
     </row>
-    <row r="65" ht="21" customHeight="1">
+    <row r="65" ht="23" customHeight="1">
       <c r="A65" s="30" t="inlineStr">
         <is>
           <t>1. 一个题型只对应一个布局值；同一枚举值在不同版本、不同等级共用同一布局。</t>
@@ -5176,7 +5178,7 @@
       <c r="F65" s="27" t="n"/>
       <c r="G65" s="27" t="n"/>
     </row>
-    <row r="66" ht="21" customHeight="1">
+    <row r="66" ht="23" customHeight="1">
       <c r="A66" s="30" t="inlineStr">
         <is>
           <t>2. choice 与 choiceGrid 的分界不是「是不是图」，而是「选项是不是同组共用的池」：图片匹配题是池 → choiceGrid；看图选择题每题自带独立三张图 → 仍是 choice。</t>
@@ -5189,7 +5191,7 @@
       <c r="F66" s="27" t="n"/>
       <c r="G66" s="27" t="n"/>
     </row>
-    <row r="67" ht="21" customHeight="1">
+    <row r="67" ht="23" customHeight="1">
       <c r="A67" s="30" t="inlineStr">
         <is>
           <t>3. shortInput 只给「答案恒为单个汉字」的题型（汉字书写）；其余文本作答一律 input，不论一行还是多行，前端按题型给字数提示。</t>
@@ -5202,7 +5204,7 @@
       <c r="F67" s="27" t="n"/>
       <c r="G67" s="27" t="n"/>
     </row>
-    <row r="68" ht="21" customHeight="1">
+    <row r="68" ht="23" customHeight="1">
       <c r="A68" s="30" t="inlineStr">
         <is>
           <t>4. multiChoice 在 HSK、HSKK 中当前无题型使用，仅 CSCA「多选」题使用（答案含逗号，如 "A,C"）；保留为合法值，不删除。</t>
@@ -5215,7 +5217,7 @@
       <c r="F68" s="27" t="n"/>
       <c r="G68" s="27" t="n"/>
     </row>
-    <row r="69" ht="21" customHeight="1">
+    <row r="69" ht="23" customHeight="1">
       <c r="A69" s="30" t="inlineStr">
         <is>
           <t>5. 图、音频、图表、表格都是「材料」，不是选项，不改变布局：只有进入选项区且同组共用时才升为 choiceGrid。</t>
@@ -5228,7 +5230,7 @@
       <c r="F69" s="27" t="n"/>
       <c r="G69" s="27" t="n"/>
     </row>
-    <row r="70" ht="21" customHeight="1">
+    <row r="70" ht="23" customHeight="1">
       <c r="A70" s="30" t="inlineStr">
         <is>
           <t>6. 布局只描述控件形态，不描述内容形式；题型的中文名与分值仍以「HSK枚举值」「HSK新旧大纲对比」两张表为准。</t>
@@ -5241,29 +5243,65 @@
       <c r="F70" s="27" t="n"/>
       <c r="G70" s="27" t="n"/>
     </row>
+    <row r="71" ht="23" customHeight="1">
+      <c r="A71" s="30" t="inlineStr">
+        <is>
+          <t>7. 若沿用旧方案（6 值：choice / judge / multiChoice / order / input / record），本表新增的 choiceGrid、shortInput 分别回退并入 choice、input，其余对应关系不变。</t>
+        </is>
+      </c>
+      <c r="B71" s="27" t="n"/>
+      <c r="C71" s="27" t="n"/>
+      <c r="D71" s="27" t="n"/>
+      <c r="E71" s="27" t="n"/>
+      <c r="F71" s="27" t="n"/>
+      <c r="G71" s="27" t="n"/>
+    </row>
+    <row r="72" ht="23" customHeight="1">
+      <c r="A72" s="30" t="inlineStr">
+        <is>
+          <t>8. 例题（example_question）不是题型、也不单独取布局值：按同卷同一题号区间的正题回填（现库 935 道例题全部可定位，无落空）。</t>
+        </is>
+      </c>
+      <c r="B72" s="27" t="n"/>
+      <c r="C72" s="27" t="n"/>
+      <c r="D72" s="27" t="n"/>
+      <c r="E72" s="27" t="n"/>
+      <c r="F72" s="27" t="n"/>
+      <c r="G72" s="27" t="n"/>
+    </row>
   </sheetData>
   <autoFilter ref="A2:G48"/>
-  <mergeCells count="20">
-    <mergeCell ref="E60:G60"/>
+  <mergeCells count="30">
+    <mergeCell ref="D60:E60"/>
+    <mergeCell ref="B54:C54"/>
+    <mergeCell ref="B59:C59"/>
+    <mergeCell ref="A72:G72"/>
+    <mergeCell ref="B56:C56"/>
+    <mergeCell ref="A61:E61"/>
     <mergeCell ref="A68:G68"/>
-    <mergeCell ref="E59:G59"/>
+    <mergeCell ref="B58:C58"/>
+    <mergeCell ref="B52:C52"/>
+    <mergeCell ref="D52:E52"/>
     <mergeCell ref="A67:G67"/>
-    <mergeCell ref="E61:G61"/>
-    <mergeCell ref="E57:G57"/>
+    <mergeCell ref="D57:E57"/>
+    <mergeCell ref="B60:C60"/>
     <mergeCell ref="A64:G64"/>
+    <mergeCell ref="B57:C57"/>
     <mergeCell ref="A51:G51"/>
-    <mergeCell ref="E54:G54"/>
+    <mergeCell ref="B53:C53"/>
+    <mergeCell ref="D53:E53"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A61:D61"/>
     <mergeCell ref="A70:G70"/>
-    <mergeCell ref="E53:G53"/>
     <mergeCell ref="A69:G69"/>
-    <mergeCell ref="E56:G56"/>
-    <mergeCell ref="E58:G58"/>
+    <mergeCell ref="D58:E58"/>
+    <mergeCell ref="D56:E56"/>
     <mergeCell ref="A65:G65"/>
-    <mergeCell ref="E55:G55"/>
+    <mergeCell ref="B55:C55"/>
     <mergeCell ref="A66:G66"/>
-    <mergeCell ref="E52:G52"/>
+    <mergeCell ref="D55:E55"/>
+    <mergeCell ref="D54:E54"/>
+    <mergeCell ref="A71:G71"/>
+    <mergeCell ref="D59:E59"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
vault backup: 2026-10-30 17:37:13
</commit_message>
<xml_diff>
--- a/02云云天平/03业务模块/HSK3.0/新旧大纲对比(含HSK、HSKK).xlsx
+++ b/02云云天平/03业务模块/HSK3.0/新旧大纲对比(含HSK、HSKK).xlsx
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="811" uniqueCount="413">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="809" uniqueCount="411">
   <si>
     <t>HSK1</t>
   </si>
@@ -662,7 +662,7 @@
     <t>出现版本-等级</t>
   </si>
   <si>
-    <t>判定依据 / 备注</t>
+    <t>备注</t>
   </si>
   <si>
     <t>看图判断题</t>
@@ -743,39 +743,36 @@
     <t>2.0 L2–L4</t>
   </si>
   <si>
+    <t>长对话选择题</t>
+  </si>
+  <si>
+    <t>listening_long_dialog_choice</t>
+  </si>
+  <si>
+    <t>对话选择题</t>
+  </si>
+  <si>
+    <t>listening_dialog_choice</t>
+  </si>
+  <si>
+    <t>3.0 L2–L4</t>
+  </si>
+  <si>
+    <t>3.0 合并短/长对话后的新名称</t>
+  </si>
+  <si>
+    <t>细节判断题</t>
+  </si>
+  <si>
+    <t>listening_detail_judge</t>
+  </si>
+  <si>
+    <t>2.0 L3、L4</t>
+  </si>
+  <si>
     <t/>
   </si>
   <si>
-    <t>长对话选择题</t>
-  </si>
-  <si>
-    <t>listening_long_dialog_choice</t>
-  </si>
-  <si>
-    <t>材料更长，控件与短对话一致</t>
-  </si>
-  <si>
-    <t>对话选择题</t>
-  </si>
-  <si>
-    <t>listening_dialog_choice</t>
-  </si>
-  <si>
-    <t>3.0 L2–L4</t>
-  </si>
-  <si>
-    <t>3.0 合并短/长对话后的新名称</t>
-  </si>
-  <si>
-    <t>细节判断题</t>
-  </si>
-  <si>
-    <t>listening_detail_judge</t>
-  </si>
-  <si>
-    <t>2.0 L3、L4</t>
-  </si>
-  <si>
     <t>阅读理解题</t>
   </si>
   <si>
@@ -806,7 +803,7 @@
     <t>listening_choice_fill</t>
   </si>
   <si>
-    <t>库内现 30 题全部为四选项单选 → 单列；若后续录入无选项的填空子题，子题改 input</t>
+    <t>四选项单选 → 单列；</t>
   </si>
   <si>
     <t>reading_judge</t>
@@ -1332,9 +1329,6 @@
   </si>
   <si>
     <t>口语（HSKK 全题型）</t>
-  </si>
-  <si>
-    <t>备注</t>
   </si>
   <si>
     <t>听一句/一段后原样复述，2.0 三档 + 3.0 三级。</t>
@@ -3858,19 +3852,17 @@
       <c r="F7" s="14" t="s">
         <v>208</v>
       </c>
-      <c r="G7" s="14" t="s">
-        <v>209</v>
-      </c>
+      <c r="G7" s="14"/>
     </row>
     <row r="8" ht="38" customHeight="1" spans="1:7">
       <c r="A8" s="13" t="s">
         <v>9</v>
       </c>
       <c r="B8" s="14" t="s">
+        <v>209</v>
+      </c>
+      <c r="C8" s="14" t="s">
         <v>210</v>
-      </c>
-      <c r="C8" s="14" t="s">
-        <v>211</v>
       </c>
       <c r="D8" s="15" t="s">
         <v>202</v>
@@ -3881,19 +3873,17 @@
       <c r="F8" s="14" t="s">
         <v>208</v>
       </c>
-      <c r="G8" s="14" t="s">
-        <v>212</v>
-      </c>
+      <c r="G8" s="14"/>
     </row>
     <row r="9" ht="23" customHeight="1" spans="1:7">
       <c r="A9" s="13" t="s">
         <v>9</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="D9" s="15" t="s">
         <v>202</v>
@@ -3902,10 +3892,10 @@
         <v>203</v>
       </c>
       <c r="F9" s="14" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="G9" s="14" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
     </row>
     <row r="10" ht="23" customHeight="1" spans="1:7">
@@ -3913,10 +3903,10 @@
         <v>9</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="D10" s="15" t="s">
         <v>185</v>
@@ -3925,10 +3915,10 @@
         <v>186</v>
       </c>
       <c r="F10" s="14" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="G10" s="14" t="s">
-        <v>209</v>
+        <v>218</v>
       </c>
     </row>
     <row r="11" ht="23" customHeight="1" spans="1:7">
@@ -3936,10 +3926,10 @@
         <v>9</v>
       </c>
       <c r="B11" s="14" t="s">
+        <v>219</v>
+      </c>
+      <c r="C11" s="14" t="s">
         <v>220</v>
-      </c>
-      <c r="C11" s="14" t="s">
-        <v>221</v>
       </c>
       <c r="D11" s="15" t="s">
         <v>202</v>
@@ -3948,10 +3938,10 @@
         <v>203</v>
       </c>
       <c r="F11" s="14" t="s">
+        <v>221</v>
+      </c>
+      <c r="G11" s="14" t="s">
         <v>222</v>
-      </c>
-      <c r="G11" s="14" t="s">
-        <v>223</v>
       </c>
     </row>
     <row r="12" ht="38" customHeight="1" spans="1:7">
@@ -3959,7 +3949,7 @@
         <v>9</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C12" s="14" t="s">
         <v>184</v>
@@ -3968,13 +3958,13 @@
         <v>185</v>
       </c>
       <c r="E12" s="14" t="s">
+        <v>224</v>
+      </c>
+      <c r="F12" s="14" t="s">
         <v>225</v>
       </c>
-      <c r="F12" s="14" t="s">
+      <c r="G12" s="14" t="s">
         <v>226</v>
-      </c>
-      <c r="G12" s="14" t="s">
-        <v>227</v>
       </c>
     </row>
     <row r="13" ht="38" customHeight="1" spans="1:7">
@@ -3982,10 +3972,10 @@
         <v>9</v>
       </c>
       <c r="B13" s="14" t="s">
+        <v>227</v>
+      </c>
+      <c r="C13" s="14" t="s">
         <v>228</v>
-      </c>
-      <c r="C13" s="14" t="s">
-        <v>229</v>
       </c>
       <c r="D13" s="15" t="s">
         <v>202</v>
@@ -3994,10 +3984,10 @@
         <v>203</v>
       </c>
       <c r="F13" s="14" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="G13" s="14" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
     </row>
     <row r="14" ht="23" customHeight="1" spans="1:7">
@@ -4008,7 +3998,7 @@
         <v>183</v>
       </c>
       <c r="C14" s="14" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="D14" s="15" t="s">
         <v>185</v>
@@ -4017,10 +4007,10 @@
         <v>186</v>
       </c>
       <c r="F14" s="14" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="G14" s="14" t="s">
-        <v>209</v>
+        <v>218</v>
       </c>
     </row>
     <row r="15" ht="23" customHeight="1" spans="1:7">
@@ -4031,7 +4021,7 @@
         <v>195</v>
       </c>
       <c r="C15" s="14" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="D15" s="15" t="s">
         <v>191</v>
@@ -4040,10 +4030,10 @@
         <v>197</v>
       </c>
       <c r="F15" s="14" t="s">
+        <v>233</v>
+      </c>
+      <c r="G15" s="14" t="s">
         <v>234</v>
-      </c>
-      <c r="G15" s="14" t="s">
-        <v>235</v>
       </c>
     </row>
     <row r="16" ht="38" customHeight="1" spans="1:7">
@@ -4051,22 +4041,22 @@
         <v>13</v>
       </c>
       <c r="B16" s="14" t="s">
+        <v>235</v>
+      </c>
+      <c r="C16" s="14" t="s">
         <v>236</v>
-      </c>
-      <c r="C16" s="14" t="s">
-        <v>237</v>
       </c>
       <c r="D16" s="15" t="s">
         <v>202</v>
       </c>
       <c r="E16" s="14" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="F16" s="14" t="s">
         <v>198</v>
       </c>
       <c r="G16" s="14" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="17" ht="38" customHeight="1" spans="1:7">
@@ -4074,22 +4064,22 @@
         <v>13</v>
       </c>
       <c r="B17" s="14" t="s">
+        <v>239</v>
+      </c>
+      <c r="C17" s="14" t="s">
         <v>240</v>
-      </c>
-      <c r="C17" s="14" t="s">
-        <v>241</v>
       </c>
       <c r="D17" s="15" t="s">
         <v>191</v>
       </c>
       <c r="E17" s="14" t="s">
+        <v>241</v>
+      </c>
+      <c r="F17" s="14" t="s">
         <v>242</v>
       </c>
-      <c r="F17" s="14" t="s">
+      <c r="G17" s="14" t="s">
         <v>243</v>
-      </c>
-      <c r="G17" s="14" t="s">
-        <v>244</v>
       </c>
     </row>
     <row r="18" ht="23" customHeight="1" spans="1:7">
@@ -4097,10 +4087,10 @@
         <v>13</v>
       </c>
       <c r="B18" s="14" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="C18" s="14" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="D18" s="15" t="s">
         <v>185</v>
@@ -4109,10 +4099,10 @@
         <v>186</v>
       </c>
       <c r="F18" s="14" t="s">
+        <v>245</v>
+      </c>
+      <c r="G18" s="14" t="s">
         <v>246</v>
-      </c>
-      <c r="G18" s="14" t="s">
-        <v>247</v>
       </c>
     </row>
     <row r="19" ht="23" customHeight="1" spans="1:7">
@@ -4123,7 +4113,7 @@
         <v>200</v>
       </c>
       <c r="C19" s="14" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="D19" s="15" t="s">
         <v>202</v>
@@ -4132,10 +4122,10 @@
         <v>203</v>
       </c>
       <c r="F19" s="14" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="G19" s="14" t="s">
-        <v>209</v>
+        <v>218</v>
       </c>
     </row>
     <row r="20" ht="38" customHeight="1" spans="1:7">
@@ -4143,22 +4133,22 @@
         <v>13</v>
       </c>
       <c r="B20" s="14" t="s">
+        <v>249</v>
+      </c>
+      <c r="C20" s="14" t="s">
         <v>250</v>
       </c>
-      <c r="C20" s="14" t="s">
+      <c r="D20" s="15" t="s">
         <v>251</v>
       </c>
-      <c r="D20" s="15" t="s">
+      <c r="E20" s="14" t="s">
         <v>252</v>
       </c>
-      <c r="E20" s="14" t="s">
+      <c r="F20" s="14" t="s">
         <v>253</v>
       </c>
-      <c r="F20" s="14" t="s">
+      <c r="G20" s="14" t="s">
         <v>254</v>
-      </c>
-      <c r="G20" s="14" t="s">
-        <v>255</v>
       </c>
     </row>
     <row r="21" ht="38" customHeight="1" spans="1:7">
@@ -4166,22 +4156,22 @@
         <v>13</v>
       </c>
       <c r="B21" s="14" t="s">
+        <v>255</v>
+      </c>
+      <c r="C21" s="14" t="s">
         <v>256</v>
-      </c>
-      <c r="C21" s="14" t="s">
-        <v>257</v>
       </c>
       <c r="D21" s="15" t="s">
         <v>202</v>
       </c>
       <c r="E21" s="14" t="s">
+        <v>257</v>
+      </c>
+      <c r="F21" s="14" t="s">
         <v>258</v>
       </c>
-      <c r="F21" s="14" t="s">
+      <c r="G21" s="14" t="s">
         <v>259</v>
-      </c>
-      <c r="G21" s="14" t="s">
-        <v>260</v>
       </c>
     </row>
     <row r="22" ht="23" customHeight="1" spans="1:7">
@@ -4189,22 +4179,22 @@
         <v>13</v>
       </c>
       <c r="B22" s="14" t="s">
+        <v>260</v>
+      </c>
+      <c r="C22" s="14" t="s">
         <v>261</v>
-      </c>
-      <c r="C22" s="14" t="s">
-        <v>262</v>
       </c>
       <c r="D22" s="15" t="s">
         <v>202</v>
       </c>
       <c r="E22" s="14" t="s">
+        <v>262</v>
+      </c>
+      <c r="F22" s="14" t="s">
         <v>263</v>
       </c>
-      <c r="F22" s="14" t="s">
+      <c r="G22" s="14" t="s">
         <v>264</v>
-      </c>
-      <c r="G22" s="14" t="s">
-        <v>265</v>
       </c>
     </row>
     <row r="23" ht="38" customHeight="1" spans="1:7">
@@ -4212,10 +4202,10 @@
         <v>13</v>
       </c>
       <c r="B23" s="14" t="s">
+        <v>265</v>
+      </c>
+      <c r="C23" s="14" t="s">
         <v>266</v>
-      </c>
-      <c r="C23" s="14" t="s">
-        <v>267</v>
       </c>
       <c r="D23" s="15" t="s">
         <v>202</v>
@@ -4224,10 +4214,10 @@
         <v>203</v>
       </c>
       <c r="F23" s="14" t="s">
+        <v>267</v>
+      </c>
+      <c r="G23" s="14" t="s">
         <v>268</v>
-      </c>
-      <c r="G23" s="14" t="s">
-        <v>269</v>
       </c>
     </row>
     <row r="24" ht="53" customHeight="1" spans="1:7">
@@ -4235,22 +4225,22 @@
         <v>13</v>
       </c>
       <c r="B24" s="14" t="s">
+        <v>269</v>
+      </c>
+      <c r="C24" s="14" t="s">
         <v>270</v>
-      </c>
-      <c r="C24" s="14" t="s">
-        <v>271</v>
       </c>
       <c r="D24" s="15" t="s">
         <v>191</v>
       </c>
       <c r="E24" s="14" t="s">
+        <v>271</v>
+      </c>
+      <c r="F24" s="14" t="s">
         <v>272</v>
       </c>
-      <c r="F24" s="14" t="s">
+      <c r="G24" s="14" t="s">
         <v>273</v>
-      </c>
-      <c r="G24" s="14" t="s">
-        <v>274</v>
       </c>
     </row>
     <row r="25" ht="38" customHeight="1" spans="1:7">
@@ -4258,22 +4248,22 @@
         <v>13</v>
       </c>
       <c r="B25" s="14" t="s">
+        <v>274</v>
+      </c>
+      <c r="C25" s="14" t="s">
         <v>275</v>
-      </c>
-      <c r="C25" s="14" t="s">
-        <v>276</v>
       </c>
       <c r="D25" s="15" t="s">
         <v>202</v>
       </c>
       <c r="E25" s="14" t="s">
+        <v>276</v>
+      </c>
+      <c r="F25" s="14" t="s">
         <v>277</v>
       </c>
-      <c r="F25" s="14" t="s">
+      <c r="G25" s="14" t="s">
         <v>278</v>
-      </c>
-      <c r="G25" s="14" t="s">
-        <v>279</v>
       </c>
     </row>
     <row r="26" ht="38" customHeight="1" spans="1:7">
@@ -4281,22 +4271,22 @@
         <v>13</v>
       </c>
       <c r="B26" s="14" t="s">
+        <v>279</v>
+      </c>
+      <c r="C26" s="14" t="s">
         <v>280</v>
-      </c>
-      <c r="C26" s="14" t="s">
-        <v>281</v>
       </c>
       <c r="D26" s="15" t="s">
         <v>191</v>
       </c>
       <c r="E26" s="14" t="s">
+        <v>281</v>
+      </c>
+      <c r="F26" s="14" t="s">
+        <v>221</v>
+      </c>
+      <c r="G26" s="14" t="s">
         <v>282</v>
-      </c>
-      <c r="F26" s="14" t="s">
-        <v>222</v>
-      </c>
-      <c r="G26" s="14" t="s">
-        <v>283</v>
       </c>
     </row>
     <row r="27" ht="38" customHeight="1" spans="1:7">
@@ -4304,512 +4294,512 @@
         <v>13</v>
       </c>
       <c r="B27" s="14" t="s">
+        <v>283</v>
+      </c>
+      <c r="C27" s="14" t="s">
         <v>284</v>
       </c>
-      <c r="C27" s="14" t="s">
+      <c r="D27" s="15" t="s">
         <v>285</v>
       </c>
-      <c r="D27" s="15" t="s">
+      <c r="E27" s="14" t="s">
         <v>286</v>
       </c>
-      <c r="E27" s="14" t="s">
+      <c r="F27" s="14" t="s">
+        <v>225</v>
+      </c>
+      <c r="G27" s="14" t="s">
         <v>287</v>
-      </c>
-      <c r="F27" s="14" t="s">
-        <v>226</v>
-      </c>
-      <c r="G27" s="14" t="s">
-        <v>288</v>
       </c>
     </row>
     <row r="28" ht="38" customHeight="1" spans="1:7">
       <c r="A28" s="13" t="s">
+        <v>288</v>
+      </c>
+      <c r="B28" s="14" t="s">
         <v>289</v>
       </c>
-      <c r="B28" s="14" t="s">
+      <c r="C28" s="14" t="s">
         <v>290</v>
       </c>
-      <c r="C28" s="14" t="s">
+      <c r="D28" s="15" t="s">
+        <v>251</v>
+      </c>
+      <c r="E28" s="14" t="s">
         <v>291</v>
       </c>
-      <c r="D28" s="15" t="s">
-        <v>252</v>
-      </c>
-      <c r="E28" s="14" t="s">
+      <c r="F28" s="14" t="s">
         <v>292</v>
       </c>
-      <c r="F28" s="14" t="s">
+      <c r="G28" s="14" t="s">
         <v>293</v>
-      </c>
-      <c r="G28" s="14" t="s">
-        <v>294</v>
       </c>
     </row>
     <row r="29" ht="38" customHeight="1" spans="1:7">
       <c r="A29" s="13" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="B29" s="14" t="s">
+        <v>294</v>
+      </c>
+      <c r="C29" s="14" t="s">
         <v>295</v>
       </c>
-      <c r="C29" s="14" t="s">
+      <c r="D29" s="15" t="s">
         <v>296</v>
       </c>
-      <c r="D29" s="15" t="s">
+      <c r="E29" s="14" t="s">
         <v>297</v>
       </c>
-      <c r="E29" s="14" t="s">
+      <c r="F29" s="14" t="s">
         <v>298</v>
       </c>
-      <c r="F29" s="14" t="s">
+      <c r="G29" s="14" t="s">
         <v>299</v>
-      </c>
-      <c r="G29" s="14" t="s">
-        <v>300</v>
       </c>
     </row>
     <row r="30" ht="38" customHeight="1" spans="1:7">
       <c r="A30" s="13" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="B30" s="14" t="s">
+        <v>300</v>
+      </c>
+      <c r="C30" s="14" t="s">
         <v>301</v>
-      </c>
-      <c r="C30" s="14" t="s">
-        <v>302</v>
       </c>
       <c r="D30" s="15" t="s">
         <v>191</v>
       </c>
       <c r="E30" s="14" t="s">
+        <v>302</v>
+      </c>
+      <c r="F30" s="14" t="s">
         <v>303</v>
       </c>
-      <c r="F30" s="14" t="s">
+      <c r="G30" s="14" t="s">
         <v>304</v>
-      </c>
-      <c r="G30" s="14" t="s">
-        <v>305</v>
       </c>
     </row>
     <row r="31" ht="23" customHeight="1" spans="1:7">
       <c r="A31" s="13" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="B31" s="14" t="s">
+        <v>305</v>
+      </c>
+      <c r="C31" s="14" t="s">
         <v>306</v>
       </c>
-      <c r="C31" s="14" t="s">
+      <c r="D31" s="15" t="s">
+        <v>285</v>
+      </c>
+      <c r="E31" s="14" t="s">
         <v>307</v>
       </c>
-      <c r="D31" s="15" t="s">
-        <v>286</v>
-      </c>
-      <c r="E31" s="14" t="s">
+      <c r="F31" s="14" t="s">
         <v>308</v>
       </c>
-      <c r="F31" s="14" t="s">
+      <c r="G31" s="14" t="s">
         <v>309</v>
-      </c>
-      <c r="G31" s="14" t="s">
-        <v>310</v>
       </c>
     </row>
     <row r="32" ht="23" customHeight="1" spans="1:7">
       <c r="A32" s="13" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="B32" s="14" t="s">
+        <v>310</v>
+      </c>
+      <c r="C32" s="14" t="s">
         <v>311</v>
       </c>
-      <c r="C32" s="14" t="s">
+      <c r="D32" s="15" t="s">
+        <v>285</v>
+      </c>
+      <c r="E32" s="14" t="s">
         <v>312</v>
       </c>
-      <c r="D32" s="15" t="s">
-        <v>286</v>
-      </c>
-      <c r="E32" s="14" t="s">
+      <c r="F32" s="14" t="s">
         <v>313</v>
       </c>
-      <c r="F32" s="14" t="s">
-        <v>314</v>
-      </c>
       <c r="G32" s="14" t="s">
-        <v>209</v>
+        <v>218</v>
       </c>
     </row>
     <row r="33" ht="23" customHeight="1" spans="1:7">
       <c r="A33" s="13" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="B33" s="14" t="s">
+        <v>314</v>
+      </c>
+      <c r="C33" s="14" t="s">
         <v>315</v>
       </c>
-      <c r="C33" s="14" t="s">
+      <c r="D33" s="15" t="s">
+        <v>285</v>
+      </c>
+      <c r="E33" s="14" t="s">
+        <v>312</v>
+      </c>
+      <c r="F33" s="14" t="s">
         <v>316</v>
       </c>
-      <c r="D33" s="15" t="s">
-        <v>286</v>
-      </c>
-      <c r="E33" s="14" t="s">
-        <v>313</v>
-      </c>
-      <c r="F33" s="14" t="s">
-        <v>317</v>
-      </c>
       <c r="G33" s="14" t="s">
-        <v>209</v>
+        <v>218</v>
       </c>
     </row>
     <row r="34" ht="23" customHeight="1" spans="1:7">
       <c r="A34" s="13" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="B34" s="14" t="s">
+        <v>317</v>
+      </c>
+      <c r="C34" s="14" t="s">
         <v>318</v>
       </c>
-      <c r="C34" s="14" t="s">
+      <c r="D34" s="15" t="s">
+        <v>285</v>
+      </c>
+      <c r="E34" s="14" t="s">
+        <v>312</v>
+      </c>
+      <c r="F34" s="14" t="s">
         <v>319</v>
       </c>
-      <c r="D34" s="15" t="s">
-        <v>286</v>
-      </c>
-      <c r="E34" s="14" t="s">
-        <v>313</v>
-      </c>
-      <c r="F34" s="14" t="s">
+      <c r="G34" s="14" t="s">
         <v>320</v>
-      </c>
-      <c r="G34" s="14" t="s">
-        <v>321</v>
       </c>
     </row>
     <row r="35" ht="23" customHeight="1" spans="1:7">
       <c r="A35" s="13" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="B35" s="14" t="s">
+        <v>321</v>
+      </c>
+      <c r="C35" s="14" t="s">
         <v>322</v>
       </c>
-      <c r="C35" s="14" t="s">
+      <c r="D35" s="15" t="s">
+        <v>285</v>
+      </c>
+      <c r="E35" s="14" t="s">
+        <v>312</v>
+      </c>
+      <c r="F35" s="14" t="s">
         <v>323</v>
       </c>
-      <c r="D35" s="15" t="s">
-        <v>286</v>
-      </c>
-      <c r="E35" s="14" t="s">
-        <v>313</v>
-      </c>
-      <c r="F35" s="14" t="s">
-        <v>324</v>
-      </c>
       <c r="G35" s="14" t="s">
-        <v>209</v>
+        <v>218</v>
       </c>
     </row>
     <row r="36" ht="23" customHeight="1" spans="1:7">
       <c r="A36" s="13" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="B36" s="14" t="s">
+        <v>324</v>
+      </c>
+      <c r="C36" s="14" t="s">
         <v>325</v>
       </c>
-      <c r="C36" s="14" t="s">
+      <c r="D36" s="15" t="s">
+        <v>285</v>
+      </c>
+      <c r="E36" s="14" t="s">
         <v>326</v>
       </c>
-      <c r="D36" s="15" t="s">
-        <v>286</v>
-      </c>
-      <c r="E36" s="14" t="s">
+      <c r="F36" s="14" t="s">
+        <v>225</v>
+      </c>
+      <c r="G36" s="14" t="s">
         <v>327</v>
-      </c>
-      <c r="F36" s="14" t="s">
-        <v>226</v>
-      </c>
-      <c r="G36" s="14" t="s">
-        <v>328</v>
       </c>
     </row>
     <row r="37" ht="23" customHeight="1" spans="1:7">
       <c r="A37" s="13" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="B37" s="14" t="s">
+        <v>328</v>
+      </c>
+      <c r="C37" s="14" t="s">
         <v>329</v>
       </c>
-      <c r="C37" s="14" t="s">
+      <c r="D37" s="15" t="s">
+        <v>285</v>
+      </c>
+      <c r="E37" s="14" t="s">
+        <v>312</v>
+      </c>
+      <c r="F37" s="14" t="s">
+        <v>277</v>
+      </c>
+      <c r="G37" s="14" t="s">
         <v>330</v>
-      </c>
-      <c r="D37" s="15" t="s">
-        <v>286</v>
-      </c>
-      <c r="E37" s="14" t="s">
-        <v>313</v>
-      </c>
-      <c r="F37" s="14" t="s">
-        <v>278</v>
-      </c>
-      <c r="G37" s="14" t="s">
-        <v>331</v>
       </c>
     </row>
     <row r="38" ht="23" customHeight="1" spans="1:7">
       <c r="A38" s="13" t="s">
+        <v>331</v>
+      </c>
+      <c r="B38" s="14" t="s">
         <v>332</v>
       </c>
-      <c r="B38" s="14" t="s">
+      <c r="C38" s="14" t="s">
         <v>333</v>
       </c>
-      <c r="C38" s="14" t="s">
-        <v>334</v>
-      </c>
       <c r="D38" s="15" t="s">
+        <v>285</v>
+      </c>
+      <c r="E38" s="14" t="s">
         <v>286</v>
       </c>
-      <c r="E38" s="14" t="s">
-        <v>287</v>
-      </c>
       <c r="F38" s="14" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="G38" s="14" t="s">
-        <v>209</v>
+        <v>218</v>
       </c>
     </row>
     <row r="39" ht="23" customHeight="1" spans="1:7">
       <c r="A39" s="13" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="B39" s="14" t="s">
+        <v>334</v>
+      </c>
+      <c r="C39" s="14" t="s">
         <v>335</v>
       </c>
-      <c r="C39" s="14" t="s">
+      <c r="D39" s="15" t="s">
         <v>336</v>
       </c>
-      <c r="D39" s="15" t="s">
+      <c r="E39" s="14" t="s">
         <v>337</v>
       </c>
-      <c r="E39" s="14" t="s">
+      <c r="F39" s="14" t="s">
+        <v>225</v>
+      </c>
+      <c r="G39" s="14" t="s">
         <v>338</v>
-      </c>
-      <c r="F39" s="14" t="s">
-        <v>226</v>
-      </c>
-      <c r="G39" s="14" t="s">
-        <v>339</v>
       </c>
     </row>
     <row r="40" ht="23" customHeight="1" spans="1:7">
       <c r="A40" s="13" t="s">
+        <v>339</v>
+      </c>
+      <c r="B40" s="14" t="s">
         <v>340</v>
       </c>
-      <c r="B40" s="14" t="s">
+      <c r="C40" s="14" t="s">
         <v>341</v>
       </c>
-      <c r="C40" s="14" t="s">
-        <v>342</v>
-      </c>
       <c r="D40" s="15" t="s">
+        <v>336</v>
+      </c>
+      <c r="E40" s="14" t="s">
         <v>337</v>
       </c>
-      <c r="E40" s="14" t="s">
-        <v>338</v>
-      </c>
       <c r="F40" s="14" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="G40" s="14" t="s">
-        <v>209</v>
+        <v>218</v>
       </c>
     </row>
     <row r="41" ht="23" customHeight="1" spans="1:7">
       <c r="A41" s="13" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="B41" s="14" t="s">
+        <v>342</v>
+      </c>
+      <c r="C41" s="14" t="s">
         <v>343</v>
       </c>
-      <c r="C41" s="14" t="s">
+      <c r="D41" s="15" t="s">
+        <v>336</v>
+      </c>
+      <c r="E41" s="14" t="s">
+        <v>337</v>
+      </c>
+      <c r="F41" s="14" t="s">
+        <v>225</v>
+      </c>
+      <c r="G41" s="14" t="s">
         <v>344</v>
-      </c>
-      <c r="D41" s="15" t="s">
-        <v>337</v>
-      </c>
-      <c r="E41" s="14" t="s">
-        <v>338</v>
-      </c>
-      <c r="F41" s="14" t="s">
-        <v>226</v>
-      </c>
-      <c r="G41" s="14" t="s">
-        <v>345</v>
       </c>
     </row>
     <row r="42" ht="23" customHeight="1" spans="1:7">
       <c r="A42" s="13" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="B42" s="14" t="s">
+        <v>345</v>
+      </c>
+      <c r="C42" s="14" t="s">
         <v>346</v>
       </c>
-      <c r="C42" s="14" t="s">
-        <v>347</v>
-      </c>
       <c r="D42" s="15" t="s">
+        <v>336</v>
+      </c>
+      <c r="E42" s="14" t="s">
         <v>337</v>
       </c>
-      <c r="E42" s="14" t="s">
-        <v>338</v>
-      </c>
       <c r="F42" s="14" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="G42" s="14" t="s">
-        <v>209</v>
+        <v>218</v>
       </c>
     </row>
     <row r="43" ht="23" customHeight="1" spans="1:7">
       <c r="A43" s="13" t="s">
+        <v>347</v>
+      </c>
+      <c r="B43" s="14" t="s">
         <v>348</v>
       </c>
-      <c r="B43" s="14" t="s">
+      <c r="C43" s="14" t="s">
         <v>349</v>
       </c>
-      <c r="C43" s="14" t="s">
+      <c r="D43" s="15" t="s">
+        <v>336</v>
+      </c>
+      <c r="E43" s="14" t="s">
+        <v>337</v>
+      </c>
+      <c r="F43" s="14" t="s">
         <v>350</v>
       </c>
-      <c r="D43" s="15" t="s">
-        <v>337</v>
-      </c>
-      <c r="E43" s="14" t="s">
-        <v>338</v>
-      </c>
-      <c r="F43" s="14" t="s">
+      <c r="G43" s="14" t="s">
         <v>351</v>
-      </c>
-      <c r="G43" s="14" t="s">
-        <v>352</v>
       </c>
     </row>
     <row r="44" ht="23" customHeight="1" spans="1:7">
       <c r="A44" s="13" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="B44" s="14" t="s">
+        <v>352</v>
+      </c>
+      <c r="C44" s="14" t="s">
         <v>353</v>
       </c>
-      <c r="C44" s="14" t="s">
+      <c r="D44" s="15" t="s">
+        <v>336</v>
+      </c>
+      <c r="E44" s="14" t="s">
+        <v>337</v>
+      </c>
+      <c r="F44" s="14" t="s">
         <v>354</v>
       </c>
-      <c r="D44" s="15" t="s">
-        <v>337</v>
-      </c>
-      <c r="E44" s="14" t="s">
-        <v>338</v>
-      </c>
-      <c r="F44" s="14" t="s">
+      <c r="G44" s="14" t="s">
         <v>355</v>
-      </c>
-      <c r="G44" s="14" t="s">
-        <v>356</v>
       </c>
     </row>
     <row r="45" ht="23" customHeight="1" spans="1:7">
       <c r="A45" s="13" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="B45" s="14" t="s">
+        <v>356</v>
+      </c>
+      <c r="C45" s="14" t="s">
         <v>357</v>
       </c>
-      <c r="C45" s="14" t="s">
+      <c r="D45" s="15" t="s">
+        <v>336</v>
+      </c>
+      <c r="E45" s="14" t="s">
+        <v>337</v>
+      </c>
+      <c r="F45" s="14" t="s">
         <v>358</v>
       </c>
-      <c r="D45" s="15" t="s">
-        <v>337</v>
-      </c>
-      <c r="E45" s="14" t="s">
-        <v>338</v>
-      </c>
-      <c r="F45" s="14" t="s">
+      <c r="G45" s="14" t="s">
         <v>359</v>
-      </c>
-      <c r="G45" s="14" t="s">
-        <v>360</v>
       </c>
     </row>
     <row r="46" ht="23" customHeight="1" spans="1:7">
       <c r="A46" s="13" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="B46" s="14" t="s">
+        <v>360</v>
+      </c>
+      <c r="C46" s="14" t="s">
         <v>361</v>
       </c>
-      <c r="C46" s="14" t="s">
+      <c r="D46" s="15" t="s">
+        <v>336</v>
+      </c>
+      <c r="E46" s="14" t="s">
+        <v>337</v>
+      </c>
+      <c r="F46" s="14" t="s">
         <v>362</v>
       </c>
-      <c r="D46" s="15" t="s">
-        <v>337</v>
-      </c>
-      <c r="E46" s="14" t="s">
-        <v>338</v>
-      </c>
-      <c r="F46" s="14" t="s">
+      <c r="G46" s="14" t="s">
         <v>363</v>
-      </c>
-      <c r="G46" s="14" t="s">
-        <v>364</v>
       </c>
     </row>
     <row r="47" ht="38" customHeight="1" spans="1:7">
       <c r="A47" s="13" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="B47" s="14" t="s">
+        <v>364</v>
+      </c>
+      <c r="C47" s="14" t="s">
         <v>365</v>
       </c>
-      <c r="C47" s="14" t="s">
+      <c r="D47" s="15" t="s">
+        <v>336</v>
+      </c>
+      <c r="E47" s="14" t="s">
+        <v>337</v>
+      </c>
+      <c r="F47" s="14" t="s">
         <v>366</v>
       </c>
-      <c r="D47" s="15" t="s">
-        <v>337</v>
-      </c>
-      <c r="E47" s="14" t="s">
-        <v>338</v>
-      </c>
-      <c r="F47" s="14" t="s">
+      <c r="G47" s="14" t="s">
         <v>367</v>
-      </c>
-      <c r="G47" s="14" t="s">
-        <v>368</v>
       </c>
     </row>
     <row r="48" ht="38" customHeight="1" spans="1:7">
       <c r="A48" s="13" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="B48" s="14" t="s">
+        <v>368</v>
+      </c>
+      <c r="C48" s="14" t="s">
         <v>369</v>
       </c>
-      <c r="C48" s="14" t="s">
+      <c r="D48" s="15" t="s">
+        <v>336</v>
+      </c>
+      <c r="E48" s="14" t="s">
+        <v>337</v>
+      </c>
+      <c r="F48" s="14" t="s">
         <v>370</v>
       </c>
-      <c r="D48" s="15" t="s">
-        <v>337</v>
-      </c>
-      <c r="E48" s="14" t="s">
-        <v>338</v>
-      </c>
-      <c r="F48" s="14" t="s">
+      <c r="G48" s="14" t="s">
         <v>371</v>
-      </c>
-      <c r="G48" s="14" t="s">
-        <v>372</v>
       </c>
     </row>
     <row r="49" ht="8" customHeight="1"/>
     <row r="50" ht="8" customHeight="1"/>
     <row r="51" ht="28" customHeight="1" spans="1:7">
       <c r="A51" s="11" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
     </row>
     <row r="52" ht="38" customHeight="1" spans="1:7">
@@ -4817,18 +4807,18 @@
         <v>179</v>
       </c>
       <c r="B52" s="12" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="C52" s="16"/>
       <c r="D52" s="12" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="E52" s="16"/>
       <c r="F52" s="12" t="s">
+        <v>375</v>
+      </c>
+      <c r="G52" s="12" t="s">
         <v>376</v>
-      </c>
-      <c r="G52" s="12" t="s">
-        <v>377</v>
       </c>
     </row>
     <row r="53" ht="38" customHeight="1" spans="1:7">
@@ -4836,18 +4826,18 @@
         <v>202</v>
       </c>
       <c r="B53" s="14" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="C53" s="17"/>
       <c r="D53" s="14" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="E53" s="17"/>
       <c r="F53" s="18">
         <v>12</v>
       </c>
       <c r="G53" s="14" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
     </row>
     <row r="54" ht="38" customHeight="1" spans="1:7">
@@ -4855,18 +4845,18 @@
         <v>191</v>
       </c>
       <c r="B54" s="14" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="C54" s="17"/>
       <c r="D54" s="14" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="E54" s="17"/>
       <c r="F54" s="18">
         <v>7</v>
       </c>
       <c r="G54" s="14" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
     </row>
     <row r="55" ht="23" customHeight="1" spans="1:7">
@@ -4874,118 +4864,118 @@
         <v>185</v>
       </c>
       <c r="B55" s="14" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="C55" s="17"/>
       <c r="D55" s="14" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="E55" s="17"/>
       <c r="F55" s="18">
         <v>5</v>
       </c>
       <c r="G55" s="14" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
     </row>
     <row r="56" ht="23" customHeight="1" spans="1:7">
       <c r="A56" s="15" t="s">
+        <v>386</v>
+      </c>
+      <c r="B56" s="14" t="s">
         <v>387</v>
-      </c>
-      <c r="B56" s="14" t="s">
-        <v>388</v>
       </c>
       <c r="C56" s="17"/>
       <c r="D56" s="14" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="E56" s="17"/>
       <c r="F56" s="18">
         <v>0</v>
       </c>
       <c r="G56" s="14" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
     </row>
     <row r="57" ht="23" customHeight="1" spans="1:7">
       <c r="A57" s="15" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="B57" s="14" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="C57" s="17"/>
       <c r="D57" s="14" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="E57" s="17"/>
       <c r="F57" s="18">
         <v>2</v>
       </c>
       <c r="G57" s="14" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
     </row>
     <row r="58" ht="23" customHeight="1" spans="1:7">
       <c r="A58" s="15" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="B58" s="14" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="C58" s="17"/>
       <c r="D58" s="14" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="E58" s="17"/>
       <c r="F58" s="18">
         <v>9</v>
       </c>
       <c r="G58" s="14" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
     </row>
     <row r="59" ht="23" customHeight="1" spans="1:7">
       <c r="A59" s="15" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="B59" s="14" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="C59" s="17"/>
       <c r="D59" s="14" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="E59" s="17"/>
       <c r="F59" s="18">
         <v>1</v>
       </c>
       <c r="G59" s="14" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="60" ht="23" customHeight="1" spans="1:7">
       <c r="A60" s="15" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="B60" s="14" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="C60" s="17"/>
       <c r="D60" s="14" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="E60" s="17"/>
       <c r="F60" s="18">
         <v>10</v>
       </c>
       <c r="G60" s="14" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
     </row>
     <row r="61" ht="24" customHeight="1" spans="1:7">
       <c r="A61" s="12" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="B61" s="16"/>
       <c r="C61" s="16"/>
@@ -5063,16 +5053,16 @@
       <c r="E1" s="2"/>
       <c r="F1" s="3"/>
       <c r="G1" s="7" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="H1" s="2"/>
       <c r="I1" s="3"/>
       <c r="J1" s="8" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="K1" s="3"/>
       <c r="L1" s="8" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="M1" s="3"/>
     </row>
@@ -5081,7 +5071,7 @@
         <v>177</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="C2" s="4" t="s">
         <v>181</v>
@@ -5090,7 +5080,7 @@
         <v>177</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="F2" s="4" t="s">
         <v>181</v>
@@ -5099,7 +5089,7 @@
         <v>177</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="I2" s="4" t="s">
         <v>181</v>
@@ -5108,13 +5098,13 @@
         <v>177</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="L2" s="4" t="s">
         <v>177</v>
       </c>
       <c r="M2" s="9" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
     </row>
     <row r="3" s="6" customFormat="1" ht="15.75" customHeight="1" spans="1:13">
@@ -5131,31 +5121,31 @@
         <v>183</v>
       </c>
       <c r="E3" s="4" t="s">
+        <v>230</v>
+      </c>
+      <c r="F3" s="4" t="s">
         <v>231</v>
       </c>
-      <c r="F3" s="4" t="s">
-        <v>232</v>
-      </c>
       <c r="G3" s="4" t="s">
+        <v>289</v>
+      </c>
+      <c r="H3" s="4" t="s">
         <v>290</v>
       </c>
-      <c r="H3" s="4" t="s">
-        <v>291</v>
-      </c>
       <c r="I3" s="4" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="J3" s="5" t="s">
+        <v>332</v>
+      </c>
+      <c r="K3" s="4" t="s">
         <v>333</v>
       </c>
-      <c r="K3" s="4" t="s">
-        <v>334</v>
-      </c>
       <c r="L3" s="5" t="s">
+        <v>340</v>
+      </c>
+      <c r="M3" s="10" t="s">
         <v>341</v>
-      </c>
-      <c r="M3" s="10" t="s">
-        <v>342</v>
       </c>
     </row>
     <row r="4" s="6" customFormat="1" ht="47.25" customHeight="1" spans="1:13">
@@ -5172,31 +5162,31 @@
         <v>195</v>
       </c>
       <c r="E4" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="F4" s="4" t="s">
         <v>233</v>
       </c>
-      <c r="F4" s="4" t="s">
-        <v>234</v>
-      </c>
       <c r="G4" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="H4" s="4" t="s">
         <v>295</v>
       </c>
-      <c r="H4" s="4" t="s">
-        <v>296</v>
-      </c>
       <c r="I4" s="4" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="J4" s="4" t="s">
+        <v>334</v>
+      </c>
+      <c r="K4" s="10" t="s">
         <v>335</v>
       </c>
-      <c r="K4" s="10" t="s">
-        <v>336</v>
-      </c>
       <c r="L4" s="10" t="s">
+        <v>342</v>
+      </c>
+      <c r="M4" s="10" t="s">
         <v>343</v>
-      </c>
-      <c r="M4" s="10" t="s">
-        <v>344</v>
       </c>
     </row>
     <row r="5" s="6" customFormat="1" ht="47.25" customHeight="1" spans="1:13">
@@ -5210,30 +5200,30 @@
         <v>198</v>
       </c>
       <c r="D5" s="4" t="s">
+        <v>235</v>
+      </c>
+      <c r="E5" s="4" t="s">
         <v>236</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>237</v>
       </c>
       <c r="F5" s="4" t="s">
         <v>198</v>
       </c>
       <c r="G5" s="4" t="s">
+        <v>300</v>
+      </c>
+      <c r="H5" s="4" t="s">
         <v>301</v>
       </c>
-      <c r="H5" s="4" t="s">
-        <v>302</v>
-      </c>
       <c r="I5" s="4" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="J5" s="10"/>
       <c r="K5" s="10"/>
       <c r="L5" s="10" t="s">
+        <v>345</v>
+      </c>
+      <c r="M5" s="10" t="s">
         <v>346</v>
-      </c>
-      <c r="M5" s="10" t="s">
-        <v>347</v>
       </c>
     </row>
     <row r="6" s="6" customFormat="1" ht="47.25" customHeight="1" spans="1:13">
@@ -5247,22 +5237,22 @@
         <v>204</v>
       </c>
       <c r="D6" s="4" t="s">
+        <v>239</v>
+      </c>
+      <c r="E6" s="4" t="s">
         <v>240</v>
       </c>
-      <c r="E6" s="4" t="s">
-        <v>241</v>
-      </c>
       <c r="F6" s="4" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="G6" s="4" t="s">
+        <v>305</v>
+      </c>
+      <c r="H6" s="4" t="s">
         <v>306</v>
       </c>
-      <c r="H6" s="4" t="s">
-        <v>307</v>
-      </c>
       <c r="I6" s="4" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="J6" s="9"/>
       <c r="K6" s="9"/>
@@ -5280,22 +5270,22 @@
         <v>208</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="G7" s="4" t="s">
+        <v>310</v>
+      </c>
+      <c r="H7" s="4" t="s">
         <v>311</v>
       </c>
-      <c r="H7" s="4" t="s">
-        <v>312</v>
-      </c>
       <c r="I7" s="4" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="J7" s="9"/>
       <c r="K7" s="9"/>
@@ -5304,10 +5294,10 @@
     </row>
     <row r="8" s="6" customFormat="1" ht="47.25" customHeight="1" spans="1:13">
       <c r="A8" s="4" t="s">
+        <v>209</v>
+      </c>
+      <c r="B8" s="4" t="s">
         <v>210</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>211</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>208</v>
@@ -5316,19 +5306,19 @@
         <v>200</v>
       </c>
       <c r="E8" s="4" t="s">
+        <v>247</v>
+      </c>
+      <c r="F8" s="4" t="s">
         <v>248</v>
       </c>
-      <c r="F8" s="4" t="s">
-        <v>249</v>
-      </c>
       <c r="G8" s="4" t="s">
+        <v>314</v>
+      </c>
+      <c r="H8" s="4" t="s">
         <v>315</v>
       </c>
-      <c r="H8" s="4" t="s">
+      <c r="I8" s="4" t="s">
         <v>316</v>
-      </c>
-      <c r="I8" s="4" t="s">
-        <v>317</v>
       </c>
       <c r="J8" s="9"/>
       <c r="K8" s="9"/>
@@ -5337,31 +5327,31 @@
     </row>
     <row r="9" s="6" customFormat="1" ht="15.75" customHeight="1" spans="1:13">
       <c r="A9" s="4" t="s">
+        <v>211</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>212</v>
+      </c>
+      <c r="C9" s="4" t="s">
         <v>213</v>
       </c>
-      <c r="B9" s="4" t="s">
-        <v>214</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>215</v>
-      </c>
       <c r="D9" s="4" t="s">
+        <v>249</v>
+      </c>
+      <c r="E9" s="4" t="s">
         <v>250</v>
       </c>
-      <c r="E9" s="4" t="s">
-        <v>251</v>
-      </c>
       <c r="F9" s="4" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="G9" s="4" t="s">
+        <v>317</v>
+      </c>
+      <c r="H9" s="4" t="s">
         <v>318</v>
       </c>
-      <c r="H9" s="4" t="s">
+      <c r="I9" s="4" t="s">
         <v>319</v>
-      </c>
-      <c r="I9" s="4" t="s">
-        <v>320</v>
       </c>
       <c r="J9" s="9"/>
       <c r="K9" s="9"/>
@@ -5370,31 +5360,31 @@
     </row>
     <row r="10" s="6" customFormat="1" ht="31.5" customHeight="1" spans="1:13">
       <c r="A10" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>216</v>
+      </c>
+      <c r="C10" s="4" t="s">
         <v>217</v>
       </c>
-      <c r="B10" s="4" t="s">
-        <v>218</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>219</v>
-      </c>
       <c r="D10" s="4" t="s">
+        <v>255</v>
+      </c>
+      <c r="E10" s="4" t="s">
         <v>256</v>
       </c>
-      <c r="E10" s="4" t="s">
-        <v>257</v>
-      </c>
       <c r="F10" s="4" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="G10" s="4" t="s">
+        <v>321</v>
+      </c>
+      <c r="H10" s="4" t="s">
         <v>322</v>
       </c>
-      <c r="H10" s="4" t="s">
+      <c r="I10" s="4" t="s">
         <v>323</v>
-      </c>
-      <c r="I10" s="4" t="s">
-        <v>324</v>
       </c>
       <c r="J10" s="9"/>
       <c r="K10" s="9"/>
@@ -5403,31 +5393,31 @@
     </row>
     <row r="11" s="6" customFormat="1" ht="31.5" customHeight="1" spans="1:13">
       <c r="A11" s="4" t="s">
+        <v>219</v>
+      </c>
+      <c r="B11" s="4" t="s">
         <v>220</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="C11" s="4" t="s">
         <v>221</v>
       </c>
-      <c r="C11" s="4" t="s">
-        <v>222</v>
-      </c>
       <c r="D11" s="4" t="s">
+        <v>260</v>
+      </c>
+      <c r="E11" s="4" t="s">
         <v>261</v>
       </c>
-      <c r="E11" s="4" t="s">
-        <v>262</v>
-      </c>
       <c r="F11" s="4" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="G11" s="4" t="s">
+        <v>324</v>
+      </c>
+      <c r="H11" s="4" t="s">
         <v>325</v>
       </c>
-      <c r="H11" s="4" t="s">
-        <v>326</v>
-      </c>
       <c r="I11" s="4" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="J11" s="9"/>
       <c r="K11" s="9"/>
@@ -5436,31 +5426,31 @@
     </row>
     <row r="12" s="6" customFormat="1" ht="47.25" customHeight="1" spans="1:13">
       <c r="A12" s="4" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B12" s="4" t="s">
         <v>184</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="D12" s="4" t="s">
+        <v>265</v>
+      </c>
+      <c r="E12" s="4" t="s">
         <v>266</v>
       </c>
-      <c r="E12" s="4" t="s">
+      <c r="F12" s="4" t="s">
         <v>267</v>
       </c>
-      <c r="F12" s="4" t="s">
-        <v>268</v>
-      </c>
       <c r="G12" s="9" t="s">
+        <v>328</v>
+      </c>
+      <c r="H12" s="9" t="s">
         <v>329</v>
       </c>
-      <c r="H12" s="9" t="s">
-        <v>330</v>
-      </c>
       <c r="I12" s="9" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="J12" s="9"/>
       <c r="K12" s="9"/>
@@ -5469,22 +5459,22 @@
     </row>
     <row r="13" s="6" customFormat="1" ht="31.5" customHeight="1" spans="1:13">
       <c r="A13" s="4" t="s">
+        <v>227</v>
+      </c>
+      <c r="B13" s="4" t="s">
         <v>228</v>
       </c>
-      <c r="B13" s="4" t="s">
-        <v>229</v>
-      </c>
       <c r="C13" s="4" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="D13" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="E13" s="4" t="s">
         <v>270</v>
       </c>
-      <c r="E13" s="4" t="s">
-        <v>271</v>
-      </c>
       <c r="F13" s="4" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="G13" s="9"/>
       <c r="H13" s="9"/>
@@ -5499,13 +5489,13 @@
       <c r="B14" s="9"/>
       <c r="C14" s="9"/>
       <c r="D14" s="4" t="s">
+        <v>274</v>
+      </c>
+      <c r="E14" s="4" t="s">
         <v>275</v>
       </c>
-      <c r="E14" s="4" t="s">
-        <v>276</v>
-      </c>
       <c r="F14" s="4" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="G14" s="9"/>
       <c r="H14" s="9"/>
@@ -5520,13 +5510,13 @@
       <c r="B15" s="9"/>
       <c r="C15" s="9"/>
       <c r="D15" s="4" t="s">
+        <v>279</v>
+      </c>
+      <c r="E15" s="4" t="s">
         <v>280</v>
       </c>
-      <c r="E15" s="4" t="s">
-        <v>281</v>
-      </c>
       <c r="F15" s="4" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="G15" s="9"/>
       <c r="H15" s="9"/>
@@ -5541,13 +5531,13 @@
       <c r="B16" s="9"/>
       <c r="C16" s="9"/>
       <c r="D16" s="4" t="s">
+        <v>283</v>
+      </c>
+      <c r="E16" s="4" t="s">
         <v>284</v>
       </c>
-      <c r="E16" s="4" t="s">
-        <v>285</v>
-      </c>
       <c r="F16" s="4" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="G16" s="9"/>
       <c r="H16" s="9"/>
@@ -5584,7 +5574,7 @@
   <sheetData>
     <row r="1" ht="22" customHeight="1" spans="1:4">
       <c r="A1" s="1" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -5595,97 +5585,97 @@
         <v>177</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="C2" s="4" t="s">
         <v>181</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>406</v>
+        <v>182</v>
       </c>
     </row>
     <row r="3" ht="34" customHeight="1" spans="1:4">
       <c r="A3" s="4" t="s">
+        <v>348</v>
+      </c>
+      <c r="B3" s="4" t="s">
         <v>349</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="C3" s="4" t="s">
         <v>350</v>
       </c>
-      <c r="C3" s="4" t="s">
-        <v>351</v>
-      </c>
       <c r="D3" s="5" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
     </row>
     <row r="4" ht="34" customHeight="1" spans="1:4">
       <c r="A4" s="4" t="s">
+        <v>352</v>
+      </c>
+      <c r="B4" s="4" t="s">
         <v>353</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="C4" s="4" t="s">
         <v>354</v>
       </c>
-      <c r="C4" s="4" t="s">
-        <v>355</v>
-      </c>
       <c r="D4" s="5" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
     </row>
     <row r="5" ht="34" customHeight="1" spans="1:4">
       <c r="A5" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="B5" s="4" t="s">
         <v>357</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="C5" s="4" t="s">
         <v>358</v>
       </c>
-      <c r="C5" s="4" t="s">
-        <v>359</v>
-      </c>
       <c r="D5" s="4" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
     </row>
     <row r="6" ht="34" customHeight="1" spans="1:4">
       <c r="A6" s="4" t="s">
+        <v>360</v>
+      </c>
+      <c r="B6" s="4" t="s">
         <v>361</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="C6" s="4" t="s">
         <v>362</v>
       </c>
-      <c r="C6" s="4" t="s">
-        <v>363</v>
-      </c>
       <c r="D6" s="4" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
     </row>
     <row r="7" ht="34" customHeight="1" spans="1:4">
       <c r="A7" s="4" t="s">
+        <v>364</v>
+      </c>
+      <c r="B7" s="4" t="s">
         <v>365</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="C7" s="4" t="s">
         <v>366</v>
       </c>
-      <c r="C7" s="4" t="s">
-        <v>367</v>
-      </c>
       <c r="D7" s="5" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
     </row>
     <row r="8" ht="34" customHeight="1" spans="1:4">
       <c r="A8" s="4" t="s">
+        <v>368</v>
+      </c>
+      <c r="B8" s="4" t="s">
         <v>369</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="C8" s="4" t="s">
         <v>370</v>
       </c>
-      <c r="C8" s="4" t="s">
-        <v>371</v>
-      </c>
       <c r="D8" s="5" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
     </row>
   </sheetData>

</xml_diff>